<commit_message>
docs: atualizar cronograma físico financeiro WAVE rev 07
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Cronograma Físico Financeiro WAVE - FIP rev 07 percentuais.xlsx
+++ b/docs/Cronograma Físico Financeiro WAVE - FIP rev 07 percentuais.xlsx
@@ -5,20 +5,17 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dasartltda.sharepoint.com/sites/DasartIncorporaes-WrEngenharia/Documentos Compartilhados/OBRAS WR/WAVE BEIRA MAR/04. ENGENHARIA/4.05 TERCEIROS/FIP INSTALAÇÕES/ARQUIVOS PARA DESENVOLVIMENTO CONTRATO/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b73f7ac4adb68b79/APP-GESTAO-CONTRATO/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="539" documentId="8_{66E8BC8A-DCAE-49C6-B59C-AFC9CA3C8614}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{08911715-F193-4453-9AD8-377C504F596B}"/>
+  <xr:revisionPtr revIDLastSave="543" documentId="8_{66E8BC8A-DCAE-49C6-B59C-AFC9CA3C8614}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{77C6BEAF-EEDB-479E-A941-60BE6F2904D8}"/>
   <bookViews>
-    <workbookView xWindow="12690" yWindow="-110" windowWidth="25820" windowHeight="10300" tabRatio="601" xr2:uid="{37B66749-6C7B-43A5-9069-298DC434CDF1}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" tabRatio="601" xr2:uid="{37B66749-6C7B-43A5-9069-298DC434CDF1}"/>
   </bookViews>
   <sheets>
     <sheet name="FÍSICO FINANCEIRO" sheetId="1" r:id="rId1"/>
     <sheet name="AUX. PAVIMENTOS" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId3"/>
-  </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'FÍSICO FINANCEIRO'!$A$3:$BB$430</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'FÍSICO FINANCEIRO'!$2:$5</definedName>
@@ -3459,353 +3456,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId3"/>
-      <xxl21:relativeUrl r:id="rId4"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="RESUMO"/>
-      <sheetName val="CR WR"/>
-      <sheetName val="MEMÓRIA ESTRUTURA"/>
-      <sheetName val="CFM - FEV 26 - VALORES"/>
-      <sheetName val="% "/>
-      <sheetName val="Avanço Percentual - Mensal"/>
-      <sheetName val="INSTALAÇÕES"/>
-      <sheetName val="Estrutura  JAN 26"/>
-      <sheetName val="Previsão Taxa WR"/>
-      <sheetName val="Estrutura"/>
-      <sheetName val="$ Estrutura"/>
-      <sheetName val="Premissas"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6">
-        <row r="4">
-          <cell r="U4">
-            <v>46142</v>
-          </cell>
-          <cell r="V4">
-            <v>46143</v>
-          </cell>
-          <cell r="W4">
-            <v>46174</v>
-          </cell>
-          <cell r="X4">
-            <v>46204</v>
-          </cell>
-          <cell r="Y4">
-            <v>46235</v>
-          </cell>
-          <cell r="Z4">
-            <v>46266</v>
-          </cell>
-          <cell r="AA4">
-            <v>46296</v>
-          </cell>
-          <cell r="AB4">
-            <v>46327</v>
-          </cell>
-          <cell r="AC4">
-            <v>46357</v>
-          </cell>
-          <cell r="AD4">
-            <v>46388</v>
-          </cell>
-          <cell r="AE4">
-            <v>46419</v>
-          </cell>
-          <cell r="AF4">
-            <v>46447</v>
-          </cell>
-          <cell r="AG4">
-            <v>46478</v>
-          </cell>
-          <cell r="AH4">
-            <v>46508</v>
-          </cell>
-          <cell r="AI4">
-            <v>46539</v>
-          </cell>
-          <cell r="AJ4">
-            <v>46569</v>
-          </cell>
-          <cell r="AK4">
-            <v>46600</v>
-          </cell>
-          <cell r="AL4">
-            <v>46632</v>
-          </cell>
-          <cell r="AM4">
-            <v>46663</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="T5" t="str">
-            <v>% FÍSICO MENSAL</v>
-          </cell>
-          <cell r="U5">
-            <v>1.2839853263295039E-3</v>
-          </cell>
-          <cell r="V5">
-            <v>3.8434671030755048E-2</v>
-          </cell>
-          <cell r="W5">
-            <v>5.2701230679677975E-2</v>
-          </cell>
-          <cell r="X5">
-            <v>7.1239900880566781E-2</v>
-          </cell>
-          <cell r="Y5">
-            <v>0.19594595001358159</v>
-          </cell>
-          <cell r="Z5">
-            <v>0.10610082012378008</v>
-          </cell>
-          <cell r="AA5">
-            <v>6.37462500861046E-2</v>
-          </cell>
-          <cell r="AB5">
-            <v>6.0131491590951547E-2</v>
-          </cell>
-          <cell r="AC5">
-            <v>5.106398997610484E-2</v>
-          </cell>
-          <cell r="AD5">
-            <v>4.5891196167568489E-2</v>
-          </cell>
-          <cell r="AE5">
-            <v>3.9571996974902594E-2</v>
-          </cell>
-          <cell r="AF5">
-            <v>3.9804733952169609E-2</v>
-          </cell>
-          <cell r="AG5">
-            <v>3.6254847154556007E-2</v>
-          </cell>
-          <cell r="AH5">
-            <v>4.8519953743070221E-2</v>
-          </cell>
-          <cell r="AI5">
-            <v>5.696557563774917E-2</v>
-          </cell>
-          <cell r="AJ5">
-            <v>4.5873059875812076E-2</v>
-          </cell>
-          <cell r="AK5">
-            <v>3.5201218031524963E-2</v>
-          </cell>
-          <cell r="AL5">
-            <v>8.1658448149772248E-3</v>
-          </cell>
-          <cell r="AM5">
-            <v>7.6983016207550592E-5</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="T6" t="str">
-            <v>% FAT. DIRETO MENSAL</v>
-          </cell>
-          <cell r="U6">
-            <v>0.16125762870275323</v>
-          </cell>
-          <cell r="V6">
-            <v>9.3347475918946085E-2</v>
-          </cell>
-          <cell r="W6">
-            <v>8.2358644072841158E-2</v>
-          </cell>
-          <cell r="X6">
-            <v>0.22419599811554547</v>
-          </cell>
-          <cell r="Y6">
-            <v>5.072565274271313E-2</v>
-          </cell>
-          <cell r="Z6">
-            <v>1.8193894407677581E-2</v>
-          </cell>
-          <cell r="AA6">
-            <v>1.3642478447611109E-2</v>
-          </cell>
-          <cell r="AB6">
-            <v>9.1732158524925278E-2</v>
-          </cell>
-          <cell r="AC6">
-            <v>0.1133125093346892</v>
-          </cell>
-          <cell r="AD6">
-            <v>1.1227524963346214E-2</v>
-          </cell>
-          <cell r="AE6">
-            <v>1.4641336627143876E-2</v>
-          </cell>
-          <cell r="AF6">
-            <v>1.790536554726093E-2</v>
-          </cell>
-          <cell r="AG6">
-            <v>2.6544159338403723E-2</v>
-          </cell>
-          <cell r="AH6">
-            <v>3.1139761591461878E-2</v>
-          </cell>
-          <cell r="AI6">
-            <v>1.1478266694668346E-2</v>
-          </cell>
-          <cell r="AJ6">
-            <v>2.4439700231891088E-2</v>
-          </cell>
-          <cell r="AK6">
-            <v>1.0299922614750705E-2</v>
-          </cell>
-          <cell r="AL6">
-            <v>3.5575221233711961E-3</v>
-          </cell>
-          <cell r="AM6">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="T7" t="str">
-            <v>%FÍSICO ACUMULADO</v>
-          </cell>
-          <cell r="U7">
-            <v>4.2924709025792488E-3</v>
-          </cell>
-          <cell r="V7">
-            <v>4.2727141933334295E-2</v>
-          </cell>
-          <cell r="W7">
-            <v>9.5428372613012263E-2</v>
-          </cell>
-          <cell r="X7">
-            <v>0.16666827349357904</v>
-          </cell>
-          <cell r="Y7">
-            <v>0.36261422350716066</v>
-          </cell>
-          <cell r="Z7">
-            <v>0.46871504363094074</v>
-          </cell>
-          <cell r="AA7">
-            <v>0.53246129371704531</v>
-          </cell>
-          <cell r="AB7">
-            <v>0.59259278530799686</v>
-          </cell>
-          <cell r="AC7">
-            <v>0.6436567752841017</v>
-          </cell>
-          <cell r="AD7">
-            <v>0.68954797145167024</v>
-          </cell>
-          <cell r="AE7">
-            <v>0.72911996842657278</v>
-          </cell>
-          <cell r="AF7">
-            <v>0.76892470237874244</v>
-          </cell>
-          <cell r="AG7">
-            <v>0.8051795495332984</v>
-          </cell>
-          <cell r="AH7">
-            <v>0.85369950327636857</v>
-          </cell>
-          <cell r="AI7">
-            <v>0.91066507891411774</v>
-          </cell>
-          <cell r="AJ7">
-            <v>0.95653813878992977</v>
-          </cell>
-          <cell r="AK7">
-            <v>0.99173935682145475</v>
-          </cell>
-          <cell r="AL7">
-            <v>0.99990520163643193</v>
-          </cell>
-          <cell r="AM7">
-            <v>0.99998218465263944</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="T8" t="str">
-            <v>% FAT. DIRETO ACUMULADO</v>
-          </cell>
-          <cell r="U8">
-            <v>0.16125762870275323</v>
-          </cell>
-          <cell r="V8">
-            <v>0.25460510462169933</v>
-          </cell>
-          <cell r="W8">
-            <v>0.33696374869454049</v>
-          </cell>
-          <cell r="X8">
-            <v>0.56115974681008596</v>
-          </cell>
-          <cell r="Y8">
-            <v>0.61188539955279908</v>
-          </cell>
-          <cell r="Z8">
-            <v>0.63007929396047668</v>
-          </cell>
-          <cell r="AA8">
-            <v>0.64372177240808781</v>
-          </cell>
-          <cell r="AB8">
-            <v>0.73545393093301303</v>
-          </cell>
-          <cell r="AC8">
-            <v>0.8487664402677022</v>
-          </cell>
-          <cell r="AD8">
-            <v>0.85999396523104843</v>
-          </cell>
-          <cell r="AE8">
-            <v>0.87463530185819227</v>
-          </cell>
-          <cell r="AF8">
-            <v>0.89254066740545324</v>
-          </cell>
-          <cell r="AG8">
-            <v>0.91908482674385694</v>
-          </cell>
-          <cell r="AH8">
-            <v>0.95022458833531886</v>
-          </cell>
-          <cell r="AI8">
-            <v>0.9617028550299872</v>
-          </cell>
-          <cell r="AJ8">
-            <v>0.98614255526187833</v>
-          </cell>
-          <cell r="AK8">
-            <v>0.99644247787662898</v>
-          </cell>
-          <cell r="AL8">
-            <v>1.0000000000000002</v>
-          </cell>
-          <cell r="AM8">
-            <v>1.0000000000000002</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
   <a:themeElements>
@@ -4134,7 +3784,7 @@
     <col min="2" max="2" width="4.7109375" style="43" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19" style="43" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8" style="43" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="73.5703125" style="55" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="54.5703125" style="55" customWidth="1"/>
     <col min="6" max="6" width="15.5703125" style="43" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="5.7109375" style="43" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="16.85546875" style="44" bestFit="1" customWidth="1"/>
@@ -49372,15 +49022,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="fd7a431a-ac48-40c9-8cfb-fb570019eb11" xsi:nil="true"/>
@@ -49389,6 +49030,15 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -49627,20 +49277,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5EB9E8F0-F327-4E84-B990-6EC8B9560054}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2F5B731-90EB-4058-9385-4A87D458D64A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="fd7a431a-ac48-40c9-8cfb-fb570019eb11"/>
     <ds:schemaRef ds:uri="c220fbd3-771c-45fb-b226-1e7078e429df"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5EB9E8F0-F327-4E84-B990-6EC8B9560054}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
feat(estrutura): métricas financeiras sob o TOTAL em todos os níveis
Novo endpoint /api/contratos/[id]/estrutura-metrics retorna por
detalhamento/tarefa/grupo:
- serviço medido (medicao_itens em medições aprovadas)
- fat. aprovados (itens_solicitacao_fat_direto aprovadas)
- NFs lançadas (notas_fiscais via medições que tocam o item)
- saldo material = subtotal_material − fat_aprovados
- saldo serviço = subtotal_mo − serviço_medido

UI: componente MetricasBloco renderiza as 5 linhas compactas abaixo
do TOTAL no header do grupo, no resumo da tarefa e ao lado de cada
detalhamento. Saldo negativo fica em vermelho.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Cronograma Físico Financeiro WAVE - FIP rev 07 percentuais.xlsx
+++ b/docs/Cronograma Físico Financeiro WAVE - FIP rev 07 percentuais.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <workbookPr codeName="EstaPastaDeTrabalho"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b73f7ac4adb68b79/APP-GESTAO-CONTRATO/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="543" documentId="8_{66E8BC8A-DCAE-49C6-B59C-AFC9CA3C8614}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{77C6BEAF-EEDB-479E-A941-60BE6F2904D8}"/>
+  <xr:revisionPtr revIDLastSave="549" documentId="8_{66E8BC8A-DCAE-49C6-B59C-AFC9CA3C8614}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{78513A6B-BE6D-45CB-80DF-2AC1A54206BD}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11040" tabRatio="601" xr2:uid="{37B66749-6C7B-43A5-9069-298DC434CDF1}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="601" xr2:uid="{37B66749-6C7B-43A5-9069-298DC434CDF1}"/>
   </bookViews>
   <sheets>
-    <sheet name="FÍSICO FINANCEIRO" sheetId="1" r:id="rId1"/>
+    <sheet name="serviço" sheetId="1" r:id="rId1"/>
     <sheet name="AUX. PAVIMENTOS" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'FÍSICO FINANCEIRO'!$A$3:$BB$430</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'FÍSICO FINANCEIRO'!$2:$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">serviço!$A$3:$BB$430</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">serviço!$2:$5</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -2926,7 +2926,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="95">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3217,9 +3217,6 @@
     <xf numFmtId="44" fontId="2" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="44" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="44" fontId="2" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3454,6 +3451,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3773,52 +3774,52 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21612B2B-65B0-4042-AF89-F6179AF39AA4}">
-  <sheetPr>
+  <sheetPr codeName="Planilha1">
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B1:BB427"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="12" outlineLevelRow="2" outlineLevelCol="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="12" outlineLevelRow="2" outlineLevelCol="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="2.42578125" style="43" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" style="43" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="2.44140625" style="43" customWidth="1"/>
+    <col min="2" max="2" width="4.6640625" style="43" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19" style="43" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8" style="43" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="54.5703125" style="55" customWidth="1"/>
-    <col min="6" max="6" width="15.5703125" style="43" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="5.7109375" style="43" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.85546875" style="44" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.42578125" style="44" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.85546875" style="44" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="5.85546875" style="43" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="12" max="12" width="10.28515625" style="45" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="13" max="13" width="9.7109375" style="45" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="14" max="14" width="11.5703125" style="45" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="15" max="15" width="9.7109375" style="45" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="16" max="16" width="9.28515625" style="45" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="17" max="17" width="10.140625" style="45" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="18" max="18" width="9.7109375" style="45" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="5" max="5" width="54.5546875" style="55" customWidth="1"/>
+    <col min="6" max="6" width="15.5546875" style="43" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.6640625" style="43" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.88671875" style="44" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.44140625" style="44" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.88671875" style="44" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="5.88671875" style="43" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="12" max="12" width="10.33203125" style="45" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="13" max="13" width="9.6640625" style="45" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="14" max="14" width="11.5546875" style="45" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="15" max="15" width="9.6640625" style="45" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="16" max="16" width="9.33203125" style="45" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="17" max="17" width="10.109375" style="45" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="18" max="18" width="9.6640625" style="45" hidden="1" customWidth="1" outlineLevel="1"/>
     <col min="19" max="19" width="10" style="45" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="20" max="20" width="10.28515625" style="45" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="21" max="21" width="10.140625" style="45" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="22" max="23" width="9.7109375" style="45" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="24" max="24" width="10.28515625" style="45" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="25" max="25" width="9.7109375" style="45" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="26" max="26" width="10.140625" style="45" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="27" max="27" width="9.7109375" style="45" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="28" max="28" width="9.28515625" style="45" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="29" max="29" width="10.140625" style="45" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="30" max="30" width="9.7109375" style="45" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="20" max="20" width="10.33203125" style="45" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="21" max="21" width="10.109375" style="45" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="22" max="23" width="9.6640625" style="45" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="24" max="24" width="10.33203125" style="45" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="25" max="25" width="9.6640625" style="45" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="26" max="26" width="10.109375" style="45" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="27" max="27" width="9.6640625" style="45" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="28" max="28" width="9.33203125" style="45" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="29" max="29" width="10.109375" style="45" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="30" max="30" width="9.6640625" style="45" hidden="1" customWidth="1" outlineLevel="1"/>
     <col min="31" max="31" width="10" style="45" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="32" max="32" width="12.7109375" style="43" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="33" max="33" width="1.7109375" style="43" customWidth="1" collapsed="1"/>
-    <col min="34" max="53" width="11.28515625" style="45" customWidth="1"/>
-    <col min="54" max="54" width="12.7109375" style="43" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="10.140625" style="43" customWidth="1"/>
-    <col min="56" max="16384" width="8.7109375" style="43"/>
+    <col min="32" max="32" width="12.6640625" style="43" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="33" max="33" width="1.6640625" style="43" customWidth="1" collapsed="1"/>
+    <col min="34" max="53" width="11.33203125" style="45" customWidth="1"/>
+    <col min="54" max="54" width="12.6640625" style="43" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="10.109375" style="43" customWidth="1"/>
+    <col min="56" max="16384" width="8.6640625" style="43"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:54" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:54" s="1" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="E1" s="47"/>
       <c r="H1" s="46">
         <f>H4/J4</f>
@@ -3924,57 +3925,57 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="2:54" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:54" s="1" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B2" s="83" t="s">
         <v>63</v>
       </c>
-      <c r="C2" s="91" t="s">
+      <c r="C2" s="90" t="s">
         <v>0</v>
       </c>
       <c r="D2" s="83" t="s">
         <v>92</v>
       </c>
-      <c r="E2" s="94" t="s">
+      <c r="E2" s="93" t="s">
         <v>801</v>
       </c>
-      <c r="F2" s="91" t="s">
-        <v>1</v>
-      </c>
-      <c r="G2" s="91" t="s">
+      <c r="F2" s="90" t="s">
+        <v>1</v>
+      </c>
+      <c r="G2" s="90" t="s">
         <v>90</v>
       </c>
-      <c r="H2" s="88" t="s">
+      <c r="H2" s="86" t="s">
         <v>61</v>
       </c>
-      <c r="I2" s="88" t="s">
+      <c r="I2" s="86" t="s">
         <v>62</v>
       </c>
       <c r="J2" s="86" t="s">
         <v>137</v>
       </c>
-      <c r="L2" s="89" t="s">
+      <c r="L2" s="88" t="s">
         <v>2</v>
       </c>
-      <c r="M2" s="89"/>
-      <c r="N2" s="89"/>
-      <c r="O2" s="89"/>
-      <c r="P2" s="89"/>
-      <c r="Q2" s="89"/>
-      <c r="R2" s="89"/>
-      <c r="S2" s="89"/>
-      <c r="T2" s="89"/>
-      <c r="U2" s="89"/>
-      <c r="V2" s="89"/>
-      <c r="W2" s="89"/>
-      <c r="X2" s="89"/>
-      <c r="Y2" s="89"/>
-      <c r="Z2" s="89"/>
-      <c r="AA2" s="89"/>
-      <c r="AB2" s="89"/>
-      <c r="AC2" s="89"/>
-      <c r="AD2" s="89"/>
-      <c r="AE2" s="89"/>
-      <c r="AF2" s="90"/>
+      <c r="M2" s="88"/>
+      <c r="N2" s="88"/>
+      <c r="O2" s="88"/>
+      <c r="P2" s="88"/>
+      <c r="Q2" s="88"/>
+      <c r="R2" s="88"/>
+      <c r="S2" s="88"/>
+      <c r="T2" s="88"/>
+      <c r="U2" s="88"/>
+      <c r="V2" s="88"/>
+      <c r="W2" s="88"/>
+      <c r="X2" s="88"/>
+      <c r="Y2" s="88"/>
+      <c r="Z2" s="88"/>
+      <c r="AA2" s="88"/>
+      <c r="AB2" s="88"/>
+      <c r="AC2" s="88"/>
+      <c r="AD2" s="88"/>
+      <c r="AE2" s="88"/>
+      <c r="AF2" s="89"/>
       <c r="AH2" s="81" t="s">
         <v>810</v>
       </c>
@@ -3999,15 +4000,15 @@
       <c r="BA2" s="81"/>
       <c r="BB2" s="82"/>
     </row>
-    <row r="3" spans="2:54" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:54" s="1" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B3" s="84"/>
-      <c r="C3" s="92"/>
+      <c r="C3" s="91"/>
       <c r="D3" s="84"/>
-      <c r="E3" s="95"/>
-      <c r="F3" s="92"/>
-      <c r="G3" s="92"/>
-      <c r="H3" s="88"/>
-      <c r="I3" s="88"/>
+      <c r="E3" s="94"/>
+      <c r="F3" s="91"/>
+      <c r="G3" s="91"/>
+      <c r="H3" s="87"/>
+      <c r="I3" s="87"/>
       <c r="J3" s="87"/>
       <c r="L3" s="3">
         <v>46111</v>
@@ -4136,13 +4137,13 @@
         <v>136</v>
       </c>
     </row>
-    <row r="4" spans="2:54" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:54" s="1" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B4" s="84"/>
-      <c r="C4" s="92"/>
+      <c r="C4" s="91"/>
       <c r="D4" s="84"/>
       <c r="E4" s="77"/>
-      <c r="F4" s="92"/>
-      <c r="G4" s="92"/>
+      <c r="F4" s="91"/>
+      <c r="G4" s="91"/>
       <c r="H4" s="86">
         <f>H7+H37+H57+H90+H139+H157+H174+H189+H211+H230+H263+H269+H280+H310+H343+H391+H407+H424</f>
         <v>11300000.001659999</v>
@@ -4324,15 +4325,15 @@
         <v>1.0000000000000002</v>
       </c>
     </row>
-    <row r="5" spans="2:54" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:54" s="1" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B5" s="85"/>
-      <c r="C5" s="93"/>
+      <c r="C5" s="92"/>
       <c r="D5" s="85"/>
       <c r="E5" s="76" t="s">
         <v>811</v>
       </c>
-      <c r="F5" s="93"/>
-      <c r="G5" s="93"/>
+      <c r="F5" s="92"/>
+      <c r="G5" s="92"/>
       <c r="H5" s="87"/>
       <c r="I5" s="87"/>
       <c r="J5" s="87"/>
@@ -4499,7 +4500,7 @@
       </c>
       <c r="BB5" s="57"/>
     </row>
-    <row r="6" spans="2:54" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:54" s="1" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B6" s="7"/>
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
@@ -4616,7 +4617,7 @@
       </c>
       <c r="BB6" s="7"/>
     </row>
-    <row r="7" spans="2:54" s="12" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:54" s="12" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B7" s="10">
         <v>1</v>
       </c>
@@ -4809,7 +4810,7 @@
         <v>1.0000000000000002</v>
       </c>
     </row>
-    <row r="8" spans="2:54" s="17" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:54" s="17" customFormat="1" ht="13.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B8" s="14">
         <v>2</v>
       </c>
@@ -5003,7 +5004,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B9" s="30">
         <v>3</v>
       </c>
@@ -5088,7 +5089,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:54" s="20" customFormat="1" ht="13.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B10" s="14">
         <v>2</v>
       </c>
@@ -5279,7 +5280,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B11" s="30">
         <v>3</v>
       </c>
@@ -5362,7 +5363,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:54" s="20" customFormat="1" ht="27.6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B12" s="14">
         <v>2</v>
       </c>
@@ -5555,7 +5556,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B13" s="30">
         <v>3</v>
       </c>
@@ -5640,7 +5641,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:54" s="20" customFormat="1" ht="27.6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B14" s="14">
         <v>2</v>
       </c>
@@ -5831,7 +5832,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:54" s="33" customFormat="1" ht="24" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B15" s="30">
         <v>3</v>
       </c>
@@ -5916,7 +5917,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:54" s="20" customFormat="1" ht="27.6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B16" s="14">
         <v>2</v>
       </c>
@@ -6107,7 +6108,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B17" s="30">
         <v>3</v>
       </c>
@@ -6192,7 +6193,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:54" s="20" customFormat="1" ht="27.6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B18" s="14">
         <v>2</v>
       </c>
@@ -6383,7 +6384,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B19" s="30">
         <v>3</v>
       </c>
@@ -6466,7 +6467,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:54" s="20" customFormat="1" ht="27.6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B20" s="14">
         <v>2</v>
       </c>
@@ -6657,7 +6658,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:54" s="33" customFormat="1" ht="24" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B21" s="30">
         <v>3</v>
       </c>
@@ -6742,7 +6743,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:54" s="20" customFormat="1" ht="13.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B22" s="14">
         <v>2</v>
       </c>
@@ -6933,7 +6934,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B23" s="30">
         <v>3</v>
       </c>
@@ -7016,7 +7017,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:54" s="20" customFormat="1" ht="27.6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B24" s="14">
         <v>2</v>
       </c>
@@ -7207,7 +7208,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B25" s="30">
         <v>3</v>
       </c>
@@ -7290,7 +7291,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:54" s="20" customFormat="1" ht="27.6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B26" s="14">
         <v>2</v>
       </c>
@@ -7481,7 +7482,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:54" s="33" customFormat="1" ht="24" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B27" s="30">
         <v>3</v>
       </c>
@@ -7566,7 +7567,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:54" s="20" customFormat="1" ht="27.6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B28" s="14">
         <v>2</v>
       </c>
@@ -7757,7 +7758,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B29" s="30">
         <v>3</v>
       </c>
@@ -7840,7 +7841,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:54" s="20" customFormat="1" ht="27.6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B30" s="14">
         <v>2</v>
       </c>
@@ -8031,7 +8032,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:54" s="33" customFormat="1" ht="24" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B31" s="30">
         <v>3</v>
       </c>
@@ -8114,7 +8115,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:54" s="20" customFormat="1" ht="13.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B32" s="14">
         <v>2</v>
       </c>
@@ -8305,7 +8306,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B33" s="30">
         <v>3</v>
       </c>
@@ -8388,7 +8389,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:54" s="20" customFormat="1" ht="27.6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B34" s="14">
         <v>2</v>
       </c>
@@ -8579,7 +8580,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:54" s="33" customFormat="1" ht="24" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B35" s="30">
         <v>3</v>
       </c>
@@ -8664,7 +8665,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="2:54" s="21" customFormat="1" ht="15" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:54" s="21" customFormat="1" ht="14.4" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B36" s="7"/>
       <c r="C36" s="7"/>
       <c r="D36" s="7"/>
@@ -8718,7 +8719,7 @@
       <c r="BA36" s="9"/>
       <c r="BB36" s="29"/>
     </row>
-    <row r="37" spans="2:54" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:54" s="1" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B37" s="10">
         <v>1</v>
       </c>
@@ -8911,7 +8912,7 @@
         <v>0.99999999999999989</v>
       </c>
     </row>
-    <row r="38" spans="2:54" s="17" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:54" s="17" customFormat="1" ht="27.6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B38" s="15">
         <v>2</v>
       </c>
@@ -9103,7 +9104,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:54" s="33" customFormat="1" ht="24" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B39" s="30">
         <v>3</v>
       </c>
@@ -9186,7 +9187,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:54" s="20" customFormat="1" ht="13.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B40" s="15">
         <v>2</v>
       </c>
@@ -9380,7 +9381,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B41" s="30">
         <v>3</v>
       </c>
@@ -9465,7 +9466,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:54" s="20" customFormat="1" ht="13.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B42" s="15">
         <v>2</v>
       </c>
@@ -9657,7 +9658,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B43" s="30">
         <v>3</v>
       </c>
@@ -9742,7 +9743,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:54" s="20" customFormat="1" ht="27.6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B44" s="15">
         <v>2</v>
       </c>
@@ -9934,7 +9935,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B45" s="30">
         <v>3</v>
       </c>
@@ -10017,7 +10018,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:54" s="20" customFormat="1" ht="27.6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B46" s="15">
         <v>2</v>
       </c>
@@ -10209,7 +10210,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:54" s="33" customFormat="1" ht="24" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B47" s="30">
         <v>3</v>
       </c>
@@ -10292,7 +10293,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:54" s="20" customFormat="1" ht="27.6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B48" s="15">
         <v>2</v>
       </c>
@@ -10484,7 +10485,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:54" s="33" customFormat="1" ht="24" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B49" s="30">
         <v>3</v>
       </c>
@@ -10567,7 +10568,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:54" s="20" customFormat="1" ht="27.6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B50" s="15">
         <v>2</v>
       </c>
@@ -10759,7 +10760,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B51" s="30">
         <v>3</v>
       </c>
@@ -10844,7 +10845,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:54" s="20" customFormat="1" ht="27.6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B52" s="15">
         <v>2</v>
       </c>
@@ -11038,7 +11039,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:54" s="33" customFormat="1" ht="24" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B53" s="30">
         <v>3</v>
       </c>
@@ -11123,7 +11124,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:54" s="20" customFormat="1" ht="13.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B54" s="15">
         <v>2</v>
       </c>
@@ -11315,7 +11316,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B55" s="30">
         <v>3</v>
       </c>
@@ -11398,7 +11399,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="2:54" s="1" customFormat="1" ht="15" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:54" s="1" customFormat="1" ht="14.4" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B56" s="7"/>
       <c r="C56" s="7"/>
       <c r="D56" s="7"/>
@@ -11452,7 +11453,7 @@
       <c r="BA56" s="9"/>
       <c r="BB56" s="7"/>
     </row>
-    <row r="57" spans="2:54" s="12" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:54" s="12" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B57" s="10">
         <v>1</v>
       </c>
@@ -11645,7 +11646,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:54" s="20" customFormat="1" ht="27.6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B58" s="15">
         <v>2</v>
       </c>
@@ -11841,7 +11842,7 @@
         <v>0.99999999999999989</v>
       </c>
     </row>
-    <row r="59" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B59" s="30">
         <v>3</v>
       </c>
@@ -11921,7 +11922,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B60" s="30">
         <v>3</v>
       </c>
@@ -12004,7 +12005,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B61" s="30">
         <v>3</v>
       </c>
@@ -12087,7 +12088,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B62" s="30">
         <v>3</v>
       </c>
@@ -12170,7 +12171,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B63" s="30">
         <v>3</v>
       </c>
@@ -12255,7 +12256,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B64" s="30">
         <v>3</v>
       </c>
@@ -12340,7 +12341,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B65" s="30">
         <v>3</v>
       </c>
@@ -12423,7 +12424,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B66" s="30">
         <v>3</v>
       </c>
@@ -12504,7 +12505,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B67" s="30">
         <v>3</v>
       </c>
@@ -12587,7 +12588,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B68" s="30">
         <v>3</v>
       </c>
@@ -12668,7 +12669,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B69" s="30">
         <v>3</v>
       </c>
@@ -12778,7 +12779,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B70" s="30">
         <v>3</v>
       </c>
@@ -12863,7 +12864,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B71" s="30">
         <v>3</v>
       </c>
@@ -12948,7 +12949,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B72" s="30">
         <v>3</v>
       </c>
@@ -13033,7 +13034,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:54" s="33" customFormat="1" ht="24" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B73" s="30">
         <v>3</v>
       </c>
@@ -13145,7 +13146,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:54" s="20" customFormat="1" ht="13.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B74" s="15">
         <v>2</v>
       </c>
@@ -13340,7 +13341,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B75" s="30">
         <v>3</v>
       </c>
@@ -13421,7 +13422,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B76" s="30">
         <v>3</v>
       </c>
@@ -13503,7 +13504,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B77" s="30">
         <v>3</v>
       </c>
@@ -13585,7 +13586,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B78" s="30">
         <v>3</v>
       </c>
@@ -13667,7 +13668,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B79" s="30">
         <v>3</v>
       </c>
@@ -13751,7 +13752,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B80" s="30">
         <v>3</v>
       </c>
@@ -13835,7 +13836,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B81" s="30">
         <v>3</v>
       </c>
@@ -13917,7 +13918,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B82" s="30">
         <v>3</v>
       </c>
@@ -13999,7 +14000,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B83" s="30">
         <v>3</v>
       </c>
@@ -14081,7 +14082,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B84" s="30">
         <v>3</v>
       </c>
@@ -14161,7 +14162,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B85" s="30">
         <v>3</v>
       </c>
@@ -14272,7 +14273,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B86" s="30">
         <v>3</v>
       </c>
@@ -14356,7 +14357,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:54" s="33" customFormat="1" ht="24" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B87" s="30">
         <v>3</v>
       </c>
@@ -14440,7 +14441,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="88" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B88" s="30">
         <v>3</v>
       </c>
@@ -14524,7 +14525,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="2:54" s="1" customFormat="1" ht="15" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:54" s="1" customFormat="1" ht="14.4" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B89" s="7"/>
       <c r="C89" s="7"/>
       <c r="D89" s="7"/>
@@ -14578,7 +14579,7 @@
       <c r="BA89" s="9"/>
       <c r="BB89" s="7"/>
     </row>
-    <row r="90" spans="2:54" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:54" s="1" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B90" s="10">
         <v>1</v>
       </c>
@@ -14777,7 +14778,7 @@
         <v>1.0000000000000002</v>
       </c>
     </row>
-    <row r="91" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:54" s="20" customFormat="1" ht="27.6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B91" s="15">
         <v>2</v>
       </c>
@@ -14964,7 +14965,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="92" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B92" s="30">
         <v>3</v>
       </c>
@@ -15047,7 +15048,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B93" s="30">
         <v>3</v>
       </c>
@@ -15132,7 +15133,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="94" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B94" s="30">
         <v>3</v>
       </c>
@@ -15217,7 +15218,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="95" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B95" s="30">
         <v>3</v>
       </c>
@@ -15302,7 +15303,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="96" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B96" s="30">
         <v>3</v>
       </c>
@@ -15387,7 +15388,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="97" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B97" s="30">
         <v>3</v>
       </c>
@@ -15472,7 +15473,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="98" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B98" s="30">
         <v>3</v>
       </c>
@@ -15557,7 +15558,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="99" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B99" s="30">
         <v>3</v>
       </c>
@@ -15642,7 +15643,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="100" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B100" s="30">
         <v>3</v>
       </c>
@@ -15728,7 +15729,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="101" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B101" s="30">
         <v>3</v>
       </c>
@@ -15813,7 +15814,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="102" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="102" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B102" s="30">
         <v>3</v>
       </c>
@@ -15923,7 +15924,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="103" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="103" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B103" s="30">
         <v>3</v>
       </c>
@@ -16010,7 +16011,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="104" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="104" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B104" s="30">
         <v>3</v>
       </c>
@@ -16097,7 +16098,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="105" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B105" s="30">
         <v>3</v>
       </c>
@@ -16184,7 +16185,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="106" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B106" s="30">
         <v>3</v>
       </c>
@@ -16271,7 +16272,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="107" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="2:54" s="20" customFormat="1" ht="27.6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B107" s="15">
         <v>2</v>
       </c>
@@ -16472,7 +16473,7 @@
         <v>0.99999999999999989</v>
       </c>
     </row>
-    <row r="108" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="108" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B108" s="30">
         <v>3</v>
       </c>
@@ -16553,7 +16554,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="109" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="109" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B109" s="30">
         <v>3</v>
       </c>
@@ -16636,7 +16637,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="110" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="110" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B110" s="30">
         <v>3</v>
       </c>
@@ -16719,7 +16720,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="111" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="111" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B111" s="30">
         <v>3</v>
       </c>
@@ -16802,7 +16803,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="112" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="112" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B112" s="30">
         <v>3</v>
       </c>
@@ -16885,7 +16886,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="113" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="113" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B113" s="30">
         <v>3</v>
       </c>
@@ -16968,7 +16969,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="114" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="114" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B114" s="30">
         <v>3</v>
       </c>
@@ -17051,7 +17052,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="115" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B115" s="30">
         <v>3</v>
       </c>
@@ -17134,7 +17135,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="116" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="116" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B116" s="30">
         <v>3</v>
       </c>
@@ -17219,7 +17220,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="117" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="117" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B117" s="30">
         <v>3</v>
       </c>
@@ -17302,7 +17303,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="118" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="118" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B118" s="30">
         <v>3</v>
       </c>
@@ -17414,7 +17415,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="119" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="119" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B119" s="30">
         <v>3</v>
       </c>
@@ -17501,7 +17502,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="120" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="120" spans="2:54" s="33" customFormat="1" ht="24" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B120" s="30">
         <v>3</v>
       </c>
@@ -17586,7 +17587,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="121" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="121" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B121" s="30">
         <v>3</v>
       </c>
@@ -17671,7 +17672,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="122" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="122" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B122" s="30">
         <v>3</v>
       </c>
@@ -17756,7 +17757,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="123" spans="2:54" s="17" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="2:54" s="17" customFormat="1" ht="27.6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B123" s="15">
         <v>2</v>
       </c>
@@ -17950,7 +17951,7 @@
         <v>1.0000000000000002</v>
       </c>
     </row>
-    <row r="124" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="124" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B124" s="30">
         <v>3</v>
       </c>
@@ -18042,7 +18043,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="125" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="125" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B125" s="30">
         <v>3</v>
       </c>
@@ -18133,7 +18134,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="126" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="126" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B126" s="30">
         <v>3</v>
       </c>
@@ -18224,7 +18225,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="127" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="127" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B127" s="30">
         <v>3</v>
       </c>
@@ -18315,7 +18316,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="128" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="128" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B128" s="30">
         <v>3</v>
       </c>
@@ -18406,7 +18407,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="129" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="129" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B129" s="30">
         <v>3</v>
       </c>
@@ -18497,7 +18498,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="130" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="130" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B130" s="30">
         <v>3</v>
       </c>
@@ -18588,7 +18589,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="131" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="131" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B131" s="30">
         <v>3</v>
       </c>
@@ -18679,7 +18680,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="132" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="132" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B132" s="30">
         <v>3</v>
       </c>
@@ -18770,7 +18771,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="133" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="133" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B133" s="30">
         <v>3</v>
       </c>
@@ -18861,7 +18862,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="134" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="134" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B134" s="30">
         <v>3</v>
       </c>
@@ -18951,7 +18952,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="135" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="135" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B135" s="30">
         <v>3</v>
       </c>
@@ -19042,7 +19043,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="136" spans="2:54" s="33" customFormat="1" ht="24" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B136" s="30">
         <v>3</v>
       </c>
@@ -19133,7 +19134,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="137" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="137" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B137" s="30">
         <v>3</v>
       </c>
@@ -19224,7 +19225,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="138" spans="2:54" s="1" customFormat="1" ht="15" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="138" spans="2:54" s="1" customFormat="1" ht="14.4" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B138" s="7"/>
       <c r="C138" s="7"/>
       <c r="D138" s="7"/>
@@ -19278,7 +19279,7 @@
       <c r="BA138" s="9"/>
       <c r="BB138" s="7"/>
     </row>
-    <row r="139" spans="2:54" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="139" spans="2:54" s="1" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B139" s="10">
         <v>1</v>
       </c>
@@ -19474,7 +19475,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="2:54" s="20" customFormat="1" ht="27.6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B140" s="15">
         <v>2</v>
       </c>
@@ -19674,7 +19675,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="141" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B141" s="30">
         <v>3</v>
       </c>
@@ -19756,7 +19757,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="142" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B142" s="30">
         <v>3</v>
       </c>
@@ -19838,7 +19839,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="143" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B143" s="30">
         <v>3</v>
       </c>
@@ -19920,7 +19921,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="144" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B144" s="30">
         <v>3</v>
       </c>
@@ -20002,7 +20003,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="145" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B145" s="30">
         <v>3</v>
       </c>
@@ -20084,7 +20085,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="146" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B146" s="30">
         <v>3</v>
       </c>
@@ -20166,7 +20167,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="147" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B147" s="30">
         <v>3</v>
       </c>
@@ -20248,7 +20249,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="148" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B148" s="30">
         <v>3</v>
       </c>
@@ -20330,7 +20331,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="149" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B149" s="30">
         <v>3</v>
       </c>
@@ -20416,7 +20417,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="150" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B150" s="30">
         <v>3</v>
       </c>
@@ -20502,7 +20503,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="151" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B151" s="30">
         <v>3</v>
       </c>
@@ -20601,7 +20602,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="152" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B152" s="30">
         <v>3</v>
       </c>
@@ -20687,7 +20688,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="153" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B153" s="30">
         <v>3</v>
       </c>
@@ -20773,7 +20774,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="154" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B154" s="30">
         <v>3</v>
       </c>
@@ -20857,7 +20858,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="155" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B155" s="30">
         <v>3</v>
       </c>
@@ -20941,7 +20942,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="2:54" s="1" customFormat="1" ht="15" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="156" spans="2:54" s="1" customFormat="1" ht="14.4" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B156" s="7"/>
       <c r="C156" s="7"/>
       <c r="D156" s="7"/>
@@ -20995,7 +20996,7 @@
       <c r="BA156" s="9"/>
       <c r="BB156" s="7"/>
     </row>
-    <row r="157" spans="2:54" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="157" spans="2:54" s="1" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B157" s="10">
         <v>1</v>
       </c>
@@ -21194,7 +21195,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="158" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="158" spans="2:54" s="20" customFormat="1" ht="13.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B158" s="15">
         <v>2</v>
       </c>
@@ -21395,7 +21396,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="159" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="159" spans="2:54" s="36" customFormat="1" ht="24" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B159" s="30">
         <v>3</v>
       </c>
@@ -21478,7 +21479,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="160" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="160" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B160" s="30">
         <v>3</v>
       </c>
@@ -21561,7 +21562,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="161" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="161" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B161" s="30">
         <v>3</v>
       </c>
@@ -21644,7 +21645,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="162" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="162" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B162" s="30">
         <v>3</v>
       </c>
@@ -21727,7 +21728,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="163" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="163" spans="2:54" s="33" customFormat="1" ht="24" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B163" s="30">
         <v>3</v>
       </c>
@@ -21810,7 +21811,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="164" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="164" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B164" s="30">
         <v>3</v>
       </c>
@@ -21893,7 +21894,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="165" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="165" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B165" s="30">
         <v>3</v>
       </c>
@@ -21976,7 +21977,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="166" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="166" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B166" s="30">
         <v>3</v>
       </c>
@@ -22059,7 +22060,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="167" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="167" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B167" s="30">
         <v>3</v>
       </c>
@@ -22142,7 +22143,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="168" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="168" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B168" s="30">
         <v>3</v>
       </c>
@@ -22225,7 +22226,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="169" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="169" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B169" s="30">
         <v>3</v>
       </c>
@@ -22329,7 +22330,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="170" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="170" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B170" s="30">
         <v>3</v>
       </c>
@@ -22414,7 +22415,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="171" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="171" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B171" s="30">
         <v>3</v>
       </c>
@@ -22499,7 +22500,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="172" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="172" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B172" s="30">
         <v>3</v>
       </c>
@@ -22584,7 +22585,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="173" spans="2:54" s="1" customFormat="1" ht="15" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="173" spans="2:54" s="1" customFormat="1" ht="14.4" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B173" s="7"/>
       <c r="C173" s="7"/>
       <c r="D173" s="7"/>
@@ -22638,7 +22639,7 @@
       <c r="BA173" s="9"/>
       <c r="BB173" s="7"/>
     </row>
-    <row r="174" spans="2:54" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="174" spans="2:54" s="1" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B174" s="10">
         <v>1</v>
       </c>
@@ -22830,7 +22831,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="175" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="175" spans="2:54" s="20" customFormat="1" ht="27.6" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B175" s="15">
         <v>2</v>
       </c>
@@ -23025,7 +23026,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="176" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="176" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B176" s="30">
         <v>3</v>
       </c>
@@ -23108,7 +23109,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="177" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="177" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B177" s="30">
         <v>3</v>
       </c>
@@ -23191,7 +23192,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="178" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="178" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B178" s="30">
         <v>3</v>
       </c>
@@ -23274,7 +23275,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="179" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="179" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B179" s="30">
         <v>3</v>
       </c>
@@ -23357,7 +23358,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="180" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="180" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B180" s="30">
         <v>3</v>
       </c>
@@ -23440,7 +23441,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="181" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="181" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B181" s="30">
         <v>3</v>
       </c>
@@ -23523,7 +23524,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="182" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="182" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B182" s="30">
         <v>3</v>
       </c>
@@ -23606,7 +23607,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="183" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="183" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B183" s="30">
         <v>3</v>
       </c>
@@ -23689,7 +23690,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="184" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="184" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B184" s="30">
         <v>3</v>
       </c>
@@ -23774,7 +23775,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="185" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="185" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B185" s="30">
         <v>3</v>
       </c>
@@ -23884,7 +23885,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="186" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="186" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B186" s="30">
         <v>3</v>
       </c>
@@ -23969,7 +23970,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="187" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="187" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B187" s="30">
         <v>3</v>
       </c>
@@ -24054,7 +24055,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="188" spans="2:54" s="1" customFormat="1" ht="15" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="188" spans="2:54" s="1" customFormat="1" ht="14.4" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B188" s="7"/>
       <c r="C188" s="7"/>
       <c r="D188" s="7"/>
@@ -24108,7 +24109,7 @@
       <c r="BA188" s="9"/>
       <c r="BB188" s="7"/>
     </row>
-    <row r="189" spans="2:54" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="189" spans="2:54" s="1" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B189" s="10">
         <v>1</v>
       </c>
@@ -24300,7 +24301,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="190" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="190" spans="2:54" s="20" customFormat="1" ht="13.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B190" s="15">
         <v>2</v>
       </c>
@@ -24495,7 +24496,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="191" spans="2:54" s="36" customFormat="1" ht="24" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="191" spans="2:54" s="36" customFormat="1" ht="24" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B191" s="30">
         <v>3</v>
       </c>
@@ -24605,7 +24606,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="192" spans="2:54" s="33" customFormat="1" ht="24" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="192" spans="2:54" s="33" customFormat="1" ht="24" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B192" s="30">
         <v>3</v>
       </c>
@@ -24688,7 +24689,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="193" spans="2:54" s="33" customFormat="1" ht="24" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="193" spans="2:54" s="33" customFormat="1" ht="24" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B193" s="30">
         <v>3</v>
       </c>
@@ -24771,7 +24772,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="194" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="194" spans="2:54" s="33" customFormat="1" ht="24" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B194" s="30">
         <v>3</v>
       </c>
@@ -24854,7 +24855,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="195" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="195" spans="2:54" s="33" customFormat="1" ht="24" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B195" s="30">
         <v>3</v>
       </c>
@@ -24937,7 +24938,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="196" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="196" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B196" s="30">
         <v>3</v>
       </c>
@@ -25022,7 +25023,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="197" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="197" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B197" s="30">
         <v>3</v>
       </c>
@@ -25105,7 +25106,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="198" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="198" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B198" s="30">
         <v>3</v>
       </c>
@@ -25190,7 +25191,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="199" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="199" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B199" s="30">
         <v>3</v>
       </c>
@@ -25273,7 +25274,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="200" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="200" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B200" s="30">
         <v>3</v>
       </c>
@@ -25358,7 +25359,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="201" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="201" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B201" s="30">
         <v>3</v>
       </c>
@@ -25443,7 +25444,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="202" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="202" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B202" s="30">
         <v>3</v>
       </c>
@@ -25526,7 +25527,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="203" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="203" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B203" s="30">
         <v>3</v>
       </c>
@@ -25634,7 +25635,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="204" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="204" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B204" s="30">
         <v>3</v>
       </c>
@@ -25717,7 +25718,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="205" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="205" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B205" s="30">
         <v>3</v>
       </c>
@@ -25800,7 +25801,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="206" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="206" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B206" s="30">
         <v>3</v>
       </c>
@@ -25883,7 +25884,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="207" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="207" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B207" s="30">
         <v>3</v>
       </c>
@@ -25966,7 +25967,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="208" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="208" spans="2:54" s="20" customFormat="1" ht="13.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B208" s="15">
         <v>2</v>
       </c>
@@ -26161,7 +26162,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="209" spans="2:54" s="36" customFormat="1" ht="24" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="209" spans="2:54" s="36" customFormat="1" ht="24" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B209" s="30">
         <v>3</v>
       </c>
@@ -26248,7 +26249,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="210" spans="2:54" s="1" customFormat="1" ht="15" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="210" spans="2:54" s="1" customFormat="1" ht="14.4" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B210" s="7"/>
       <c r="C210" s="7"/>
       <c r="D210" s="7"/>
@@ -26302,7 +26303,7 @@
       <c r="BA210" s="9"/>
       <c r="BB210" s="7"/>
     </row>
-    <row r="211" spans="2:54" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="211" spans="2:54" s="1" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B211" s="10">
         <v>1</v>
       </c>
@@ -26494,7 +26495,7 @@
         <v>1.0000000000000002</v>
       </c>
     </row>
-    <row r="212" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="212" spans="2:54" s="20" customFormat="1" ht="13.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B212" s="15">
         <v>2</v>
       </c>
@@ -26689,7 +26690,7 @@
         <v>1.0000000000000002</v>
       </c>
     </row>
-    <row r="213" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="213" spans="2:54" s="36" customFormat="1" ht="24" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B213" s="30">
         <v>3</v>
       </c>
@@ -26799,7 +26800,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="214" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="214" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B214" s="30">
         <v>3</v>
       </c>
@@ -26882,7 +26883,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="215" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="215" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B215" s="30">
         <v>3</v>
       </c>
@@ -26965,7 +26966,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="216" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="216" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B216" s="30">
         <v>3</v>
       </c>
@@ -27048,7 +27049,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="217" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="217" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B217" s="30">
         <v>3</v>
       </c>
@@ -27131,7 +27132,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="218" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="218" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B218" s="30">
         <v>3</v>
       </c>
@@ -27216,7 +27217,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="219" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="219" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B219" s="30">
         <v>3</v>
       </c>
@@ -27299,7 +27300,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="220" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="220" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B220" s="30">
         <v>3</v>
       </c>
@@ -27384,7 +27385,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="221" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="221" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B221" s="30">
         <v>3</v>
       </c>
@@ -27467,7 +27468,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="222" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="222" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B222" s="30">
         <v>3</v>
       </c>
@@ -27552,7 +27553,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="223" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="223" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B223" s="30">
         <v>3</v>
       </c>
@@ -27637,7 +27638,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="224" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="224" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B224" s="30">
         <v>3</v>
       </c>
@@ -27720,7 +27721,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="225" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="225" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B225" s="30">
         <v>3</v>
       </c>
@@ -27832,7 +27833,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="226" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="226" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B226" s="30">
         <v>3</v>
       </c>
@@ -27917,7 +27918,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="227" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="227" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B227" s="30">
         <v>3</v>
       </c>
@@ -28002,7 +28003,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="228" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="228" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B228" s="30">
         <v>3</v>
       </c>
@@ -28087,7 +28088,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="229" spans="2:54" s="1" customFormat="1" ht="15" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="229" spans="2:54" s="1" customFormat="1" ht="14.4" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B229" s="7"/>
       <c r="C229" s="7"/>
       <c r="D229" s="7"/>
@@ -28141,7 +28142,7 @@
       <c r="BA229" s="9"/>
       <c r="BB229" s="7"/>
     </row>
-    <row r="230" spans="2:54" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="230" spans="2:54" s="1" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B230" s="10">
         <v>1</v>
       </c>
@@ -28339,7 +28340,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="231" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="231" spans="2:54" s="20" customFormat="1" ht="13.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B231" s="15">
         <v>2</v>
       </c>
@@ -28534,7 +28535,7 @@
         <v>0.99999999999999978</v>
       </c>
     </row>
-    <row r="232" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="232" spans="2:54" s="36" customFormat="1" ht="24" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B232" s="30">
         <v>3</v>
       </c>
@@ -28644,7 +28645,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="233" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="233" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B233" s="30">
         <v>3</v>
       </c>
@@ -28727,7 +28728,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="234" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="234" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B234" s="30">
         <v>3</v>
       </c>
@@ -28810,7 +28811,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="235" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="235" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B235" s="30">
         <v>3</v>
       </c>
@@ -28893,7 +28894,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="236" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="236" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B236" s="30">
         <v>3</v>
       </c>
@@ -28976,7 +28977,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="237" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="237" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B237" s="30">
         <v>3</v>
       </c>
@@ -29061,7 +29062,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="238" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="238" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B238" s="30">
         <v>3</v>
       </c>
@@ -29134,7 +29135,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="239" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="239" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B239" s="30">
         <v>3</v>
       </c>
@@ -29219,7 +29220,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="240" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="240" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B240" s="30">
         <v>3</v>
       </c>
@@ -29302,7 +29303,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="241" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="241" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B241" s="30">
         <v>3</v>
       </c>
@@ -29387,7 +29388,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="242" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="242" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B242" s="30">
         <v>3</v>
       </c>
@@ -29472,7 +29473,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="243" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="243" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B243" s="30">
         <v>3</v>
       </c>
@@ -29584,7 +29585,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="244" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="244" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B244" s="30">
         <v>3</v>
       </c>
@@ -29669,7 +29670,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="245" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="245" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B245" s="30">
         <v>3</v>
       </c>
@@ -29754,7 +29755,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="246" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="246" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B246" s="30">
         <v>3</v>
       </c>
@@ -29839,7 +29840,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="247" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="247" spans="2:54" s="20" customFormat="1" ht="13.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B247" s="15">
         <v>2</v>
       </c>
@@ -30034,7 +30035,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="248" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="248" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B248" s="66">
         <v>3</v>
       </c>
@@ -30146,7 +30147,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="249" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="249" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B249" s="66">
         <v>3</v>
       </c>
@@ -30232,7 +30233,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="250" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="250" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B250" s="66">
         <v>3</v>
       </c>
@@ -30317,7 +30318,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="251" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="251" spans="2:54" s="20" customFormat="1" ht="13.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B251" s="15">
         <v>2</v>
       </c>
@@ -30512,7 +30513,7 @@
         <v>1.0000000000000002</v>
       </c>
     </row>
-    <row r="252" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="252" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B252" s="30">
         <v>3</v>
       </c>
@@ -30613,7 +30614,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="253" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="253" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B253" s="30">
         <v>3</v>
       </c>
@@ -30697,7 +30698,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="254" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="254" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B254" s="30">
         <v>3</v>
       </c>
@@ -30781,7 +30782,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="255" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="255" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B255" s="30">
         <v>3</v>
       </c>
@@ -30868,7 +30869,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="256" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="256" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B256" s="30">
         <v>3</v>
       </c>
@@ -30955,7 +30956,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="257" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="257" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B257" s="30">
         <v>3</v>
       </c>
@@ -31041,7 +31042,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="258" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="258" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B258" s="30">
         <v>3</v>
       </c>
@@ -31128,7 +31129,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="259" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="259" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B259" s="30">
         <v>3</v>
       </c>
@@ -31215,7 +31216,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="260" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="260" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B260" s="30">
         <v>3</v>
       </c>
@@ -31302,7 +31303,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="261" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="261" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B261" s="30">
         <v>3</v>
       </c>
@@ -31389,7 +31390,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="262" spans="2:54" s="1" customFormat="1" ht="15" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="262" spans="2:54" s="1" customFormat="1" ht="14.4" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B262" s="7"/>
       <c r="C262" s="7"/>
       <c r="D262" s="7"/>
@@ -31443,7 +31444,7 @@
       <c r="BA262" s="9"/>
       <c r="BB262" s="7"/>
     </row>
-    <row r="263" spans="2:54" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="263" spans="2:54" s="1" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B263" s="10">
         <v>1</v>
       </c>
@@ -31635,7 +31636,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="264" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="264" spans="2:54" s="20" customFormat="1" ht="13.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B264" s="15">
         <v>2</v>
       </c>
@@ -31828,7 +31829,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="265" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="265" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B265" s="30">
         <v>3</v>
       </c>
@@ -31917,7 +31918,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="266" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="266" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B266" s="30">
         <v>3</v>
       </c>
@@ -32002,7 +32003,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="267" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="267" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B267" s="30">
         <v>3</v>
       </c>
@@ -32088,7 +32089,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="268" spans="2:54" s="1" customFormat="1" ht="15" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="268" spans="2:54" s="1" customFormat="1" ht="14.4" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B268" s="7"/>
       <c r="C268" s="7"/>
       <c r="D268" s="7"/>
@@ -32142,7 +32143,7 @@
       <c r="BA268" s="9"/>
       <c r="BB268" s="7"/>
     </row>
-    <row r="269" spans="2:54" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="269" spans="2:54" s="1" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B269" s="10">
         <v>1</v>
       </c>
@@ -32334,7 +32335,7 @@
         <v>0.99999999999999989</v>
       </c>
     </row>
-    <row r="270" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="270" spans="2:54" s="20" customFormat="1" ht="13.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B270" s="15">
         <v>2</v>
       </c>
@@ -32528,7 +32529,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="271" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="271" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B271" s="30">
         <v>3</v>
       </c>
@@ -32618,7 +32619,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="272" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="272" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B272" s="30">
         <v>3</v>
       </c>
@@ -32708,7 +32709,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="273" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="273" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B273" s="30">
         <v>3</v>
       </c>
@@ -32798,7 +32799,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="274" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="274" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B274" s="30">
         <v>3</v>
       </c>
@@ -32884,7 +32885,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="275" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="275" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B275" s="30">
         <v>3</v>
       </c>
@@ -32968,7 +32969,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="276" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="276" spans="2:54" s="20" customFormat="1" ht="13.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B276" s="15">
         <v>2</v>
       </c>
@@ -33161,7 +33162,7 @@
         <v>0.99999999999999989</v>
       </c>
     </row>
-    <row r="277" spans="2:54" s="36" customFormat="1" ht="13.5" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="277" spans="2:54" s="36" customFormat="1" ht="13.8" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B277" s="30">
         <v>3</v>
       </c>
@@ -33265,7 +33266,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="278" spans="2:54" s="33" customFormat="1" ht="13.5" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="278" spans="2:54" s="33" customFormat="1" ht="13.8" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B278" s="30">
         <v>3</v>
       </c>
@@ -33352,7 +33353,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="279" spans="2:54" s="1" customFormat="1" ht="15" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="279" spans="2:54" s="1" customFormat="1" ht="14.4" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B279" s="7"/>
       <c r="C279" s="7"/>
       <c r="D279" s="7"/>
@@ -33406,7 +33407,7 @@
       <c r="BA279" s="9"/>
       <c r="BB279" s="7"/>
     </row>
-    <row r="280" spans="2:54" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="280" spans="2:54" s="1" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B280" s="10">
         <v>1</v>
       </c>
@@ -33599,7 +33600,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="281" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="281" spans="2:54" s="20" customFormat="1" ht="13.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B281" s="15">
         <v>2</v>
       </c>
@@ -33795,7 +33796,7 @@
         <v>0.99999999999999989</v>
       </c>
     </row>
-    <row r="282" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="282" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B282" s="30">
         <v>3</v>
       </c>
@@ -33908,7 +33909,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="283" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="283" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B283" s="30">
         <v>3</v>
       </c>
@@ -34021,7 +34022,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="284" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="284" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B284" s="30">
         <v>3</v>
       </c>
@@ -34107,7 +34108,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="285" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="285" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B285" s="30">
         <v>3</v>
       </c>
@@ -34193,7 +34194,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="286" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="286" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B286" s="30">
         <v>3</v>
       </c>
@@ -34279,7 +34280,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="287" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="287" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B287" s="30">
         <v>3</v>
       </c>
@@ -34392,7 +34393,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="288" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="288" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B288" s="30">
         <v>3</v>
       </c>
@@ -34479,7 +34480,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="289" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="289" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B289" s="30">
         <v>3</v>
       </c>
@@ -34566,7 +34567,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="290" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="290" spans="2:54" s="20" customFormat="1" ht="13.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B290" s="15">
         <v>2</v>
       </c>
@@ -34761,7 +34762,7 @@
         <v>0.99999999999999956</v>
       </c>
     </row>
-    <row r="291" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="291" spans="2:54" s="36" customFormat="1" ht="24" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B291" s="30">
         <v>3</v>
       </c>
@@ -34900,7 +34901,7 @@
         <v>0.99999999999999978</v>
       </c>
     </row>
-    <row r="292" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="292" spans="2:54" s="33" customFormat="1" ht="24" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B292" s="30">
         <v>3</v>
       </c>
@@ -34987,7 +34988,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="293" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="293" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B293" s="30">
         <v>3</v>
       </c>
@@ -35076,7 +35077,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="294" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="294" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B294" s="30">
         <v>3</v>
       </c>
@@ -35165,7 +35166,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="295" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="295" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B295" s="30">
         <v>3</v>
       </c>
@@ -35254,7 +35255,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="296" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="296" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B296" s="30">
         <v>3</v>
       </c>
@@ -35343,7 +35344,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="297" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="297" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B297" s="30">
         <v>3</v>
       </c>
@@ -35431,7 +35432,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="298" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="298" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B298" s="30">
         <v>3</v>
       </c>
@@ -35520,7 +35521,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="299" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="299" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B299" s="30">
         <v>3</v>
       </c>
@@ -35609,7 +35610,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="300" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="300" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B300" s="30">
         <v>3</v>
       </c>
@@ -35698,7 +35699,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="301" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="301" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B301" s="30">
         <v>3</v>
       </c>
@@ -35785,7 +35786,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="302" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="302" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B302" s="30">
         <v>3</v>
       </c>
@@ -35874,7 +35875,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="303" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="303" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B303" s="30">
         <v>3</v>
       </c>
@@ -36014,7 +36015,7 @@
         <v>1.0000000000000004</v>
       </c>
     </row>
-    <row r="304" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="304" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B304" s="30">
         <v>3</v>
       </c>
@@ -36100,7 +36101,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="305" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="305" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B305" s="30">
         <v>3</v>
       </c>
@@ -36186,7 +36187,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="306" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="306" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B306" s="30">
         <v>3</v>
       </c>
@@ -36272,7 +36273,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="307" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="307" spans="2:54" s="20" customFormat="1" ht="13.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B307" s="15">
         <v>2</v>
       </c>
@@ -36467,7 +36468,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="308" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="308" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B308" s="30">
         <v>3</v>
       </c>
@@ -36554,7 +36555,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="309" spans="2:54" s="1" customFormat="1" ht="15" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="309" spans="2:54" s="1" customFormat="1" ht="14.4" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B309" s="7"/>
       <c r="C309" s="7"/>
       <c r="D309" s="7"/>
@@ -36608,7 +36609,7 @@
       <c r="BA309" s="9"/>
       <c r="BB309" s="7"/>
     </row>
-    <row r="310" spans="2:54" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="310" spans="2:54" s="1" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B310" s="10">
         <v>1</v>
       </c>
@@ -36806,7 +36807,7 @@
         <v>1.0000000000000004</v>
       </c>
     </row>
-    <row r="311" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="311" spans="2:54" s="20" customFormat="1" ht="13.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B311" s="15">
         <v>2</v>
       </c>
@@ -37005,7 +37006,7 @@
         <v>0.99999999999999989</v>
       </c>
     </row>
-    <row r="312" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="312" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B312" s="30">
         <v>3</v>
       </c>
@@ -37090,7 +37091,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="313" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="313" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B313" s="30">
         <v>3</v>
       </c>
@@ -37175,7 +37176,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="314" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="314" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B314" s="30">
         <v>3</v>
       </c>
@@ -37260,7 +37261,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="315" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="315" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B315" s="30">
         <v>3</v>
       </c>
@@ -37345,7 +37346,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="316" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="316" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B316" s="30">
         <v>3</v>
       </c>
@@ -37430,7 +37431,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="317" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="317" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B317" s="30">
         <v>3</v>
       </c>
@@ -37515,7 +37516,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="318" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="318" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B318" s="30">
         <v>3</v>
       </c>
@@ -37600,7 +37601,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="319" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="319" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B319" s="30">
         <v>3</v>
       </c>
@@ -37685,7 +37686,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="320" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="320" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B320" s="30">
         <v>3</v>
       </c>
@@ -37770,7 +37771,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="321" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="321" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B321" s="30">
         <v>3</v>
       </c>
@@ -37855,7 +37856,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="322" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="322" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B322" s="30">
         <v>3</v>
       </c>
@@ -37939,7 +37940,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="323" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="323" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B323" s="30">
         <v>3</v>
       </c>
@@ -38024,7 +38025,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="324" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="324" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B324" s="30">
         <v>3</v>
       </c>
@@ -38109,7 +38110,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="325" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="325" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B325" s="30">
         <v>3</v>
       </c>
@@ -38194,7 +38195,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="326" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="326" spans="2:54" s="20" customFormat="1" ht="13.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B326" s="15">
         <v>2</v>
       </c>
@@ -38395,7 +38396,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="327" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="327" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B327" s="30">
         <v>3</v>
       </c>
@@ -38480,7 +38481,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="328" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="328" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B328" s="30">
         <v>3</v>
       </c>
@@ -38565,7 +38566,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="329" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="329" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B329" s="30">
         <v>3</v>
       </c>
@@ -38650,7 +38651,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="330" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="330" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B330" s="30">
         <v>3</v>
       </c>
@@ -38735,7 +38736,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="331" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="331" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B331" s="30">
         <v>3</v>
       </c>
@@ -38820,7 +38821,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="332" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="332" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B332" s="30">
         <v>3</v>
       </c>
@@ -38905,7 +38906,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="333" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="333" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B333" s="30">
         <v>3</v>
       </c>
@@ -38990,7 +38991,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="334" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="334" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B334" s="30">
         <v>3</v>
       </c>
@@ -39075,7 +39076,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="335" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="335" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B335" s="30">
         <v>3</v>
       </c>
@@ -39160,7 +39161,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="336" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="336" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B336" s="30">
         <v>3</v>
       </c>
@@ -39245,7 +39246,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="337" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="337" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B337" s="30">
         <v>3</v>
       </c>
@@ -39331,7 +39332,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="338" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="338" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B338" s="30">
         <v>3</v>
       </c>
@@ -39416,7 +39417,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="339" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="339" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B339" s="30">
         <v>3</v>
       </c>
@@ -39501,7 +39502,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="340" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="340" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B340" s="30">
         <v>3</v>
       </c>
@@ -39586,7 +39587,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="341" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="341" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B341" s="30">
         <v>3</v>
       </c>
@@ -39671,7 +39672,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="342" spans="2:54" s="21" customFormat="1" ht="15" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="342" spans="2:54" s="21" customFormat="1" ht="14.4" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B342" s="25"/>
       <c r="C342" s="25"/>
       <c r="D342" s="25"/>
@@ -39724,7 +39725,7 @@
       <c r="BA342" s="29"/>
       <c r="BB342" s="29"/>
     </row>
-    <row r="343" spans="2:54" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="343" spans="2:54" s="1" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B343" s="10">
         <v>1</v>
       </c>
@@ -39922,7 +39923,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="344" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="344" spans="2:54" s="20" customFormat="1" ht="13.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B344" s="15">
         <v>2</v>
       </c>
@@ -40122,7 +40123,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="345" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="345" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B345" s="30">
         <v>3</v>
       </c>
@@ -40206,7 +40207,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="346" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="346" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B346" s="30">
         <v>3</v>
       </c>
@@ -40290,7 +40291,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="347" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="347" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B347" s="30">
         <v>3</v>
       </c>
@@ -40374,7 +40375,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="348" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="348" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B348" s="30">
         <v>3</v>
       </c>
@@ -40458,7 +40459,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="349" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="349" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B349" s="30">
         <v>3</v>
       </c>
@@ -40542,7 +40543,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="350" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="350" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B350" s="30">
         <v>3</v>
       </c>
@@ -40626,7 +40627,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="351" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="351" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B351" s="30">
         <v>3</v>
       </c>
@@ -40710,7 +40711,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="352" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="352" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B352" s="30">
         <v>3</v>
       </c>
@@ -40794,7 +40795,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="353" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="353" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B353" s="30">
         <v>3</v>
       </c>
@@ -40880,7 +40881,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="354" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="354" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B354" s="30">
         <v>3</v>
       </c>
@@ -40966,7 +40967,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="355" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="355" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B355" s="30">
         <v>3</v>
       </c>
@@ -41075,7 +41076,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="356" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="356" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B356" s="30">
         <v>3</v>
       </c>
@@ -41161,7 +41162,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="357" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="357" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B357" s="30">
         <v>3</v>
       </c>
@@ -41247,7 +41248,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="358" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="358" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B358" s="30">
         <v>3</v>
       </c>
@@ -41333,7 +41334,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="359" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="359" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B359" s="30">
         <v>3</v>
       </c>
@@ -41444,7 +41445,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="360" spans="2:54" s="17" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="360" spans="2:54" s="17" customFormat="1" ht="13.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B360" s="15">
         <v>2</v>
       </c>
@@ -41644,7 +41645,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="361" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="361" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B361" s="30">
         <v>3</v>
       </c>
@@ -41727,7 +41728,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="362" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="362" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B362" s="30">
         <v>3</v>
       </c>
@@ -41810,7 +41811,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="363" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="363" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B363" s="30">
         <v>3</v>
       </c>
@@ -41893,7 +41894,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="364" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="364" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B364" s="30">
         <v>3</v>
       </c>
@@ -41976,7 +41977,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="365" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="365" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B365" s="30">
         <v>3</v>
       </c>
@@ -42059,7 +42060,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="366" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="366" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B366" s="30">
         <v>3</v>
       </c>
@@ -42142,7 +42143,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="367" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="367" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B367" s="30">
         <v>3</v>
       </c>
@@ -42225,7 +42226,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="368" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="368" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B368" s="30">
         <v>3</v>
       </c>
@@ -42308,7 +42309,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="369" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="369" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B369" s="30">
         <v>3</v>
       </c>
@@ -42393,7 +42394,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="370" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="370" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B370" s="30">
         <v>3</v>
       </c>
@@ -42476,7 +42477,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="371" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="371" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B371" s="30">
         <v>3</v>
       </c>
@@ -42586,7 +42587,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="372" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="372" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B372" s="30">
         <v>3</v>
       </c>
@@ -42671,7 +42672,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="373" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="373" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B373" s="30">
         <v>3</v>
       </c>
@@ -42756,7 +42757,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="374" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="374" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B374" s="30">
         <v>3</v>
       </c>
@@ -42841,7 +42842,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="375" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="375" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B375" s="30">
         <v>3</v>
       </c>
@@ -42949,7 +42950,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="376" spans="2:54" s="17" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="376" spans="2:54" s="17" customFormat="1" ht="13.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B376" s="15">
         <v>2</v>
       </c>
@@ -43148,7 +43149,7 @@
         <v>0.99999999999999989</v>
       </c>
     </row>
-    <row r="377" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="377" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B377" s="30">
         <v>3</v>
       </c>
@@ -43235,7 +43236,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="378" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="378" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B378" s="30">
         <v>3</v>
       </c>
@@ -43322,7 +43323,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="379" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="379" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B379" s="30">
         <v>3</v>
       </c>
@@ -43409,7 +43410,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="380" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="380" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B380" s="30">
         <v>3</v>
       </c>
@@ -43496,7 +43497,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="381" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="381" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B381" s="30">
         <v>3</v>
       </c>
@@ -43583,7 +43584,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="382" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="382" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B382" s="30">
         <v>3</v>
       </c>
@@ -43670,7 +43671,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="383" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="383" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B383" s="30">
         <v>3</v>
       </c>
@@ -43757,7 +43758,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="384" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="384" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B384" s="30">
         <v>3</v>
       </c>
@@ -43844,7 +43845,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="385" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="385" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B385" s="30">
         <v>3</v>
       </c>
@@ -43931,7 +43932,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="386" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="386" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B386" s="30">
         <v>3</v>
       </c>
@@ -44018,7 +44019,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="387" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="387" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B387" s="30">
         <v>3</v>
       </c>
@@ -44110,7 +44111,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="388" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="388" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B388" s="30">
         <v>3</v>
       </c>
@@ -44197,7 +44198,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="389" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="389" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B389" s="30">
         <v>3</v>
       </c>
@@ -44285,7 +44286,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="390" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="390" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B390" s="30">
         <v>3</v>
       </c>
@@ -44373,7 +44374,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="391" spans="2:54" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="391" spans="2:54" s="1" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B391" s="10">
         <v>1</v>
       </c>
@@ -44565,7 +44566,7 @@
         <v>0.99999999999999989</v>
       </c>
     </row>
-    <row r="392" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="392" spans="2:54" s="20" customFormat="1" ht="13.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B392" s="15">
         <v>2</v>
       </c>
@@ -44759,7 +44760,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="393" spans="2:54" s="36" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="393" spans="2:54" s="36" customFormat="1" ht="24" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B393" s="30">
         <v>3</v>
       </c>
@@ -44869,7 +44870,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="394" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="394" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B394" s="30">
         <v>3</v>
       </c>
@@ -44955,7 +44956,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="395" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="395" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B395" s="30">
         <v>3</v>
       </c>
@@ -45041,7 +45042,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="396" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="396" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B396" s="30">
         <v>3</v>
       </c>
@@ -45129,7 +45130,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="397" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="397" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B397" s="30">
         <v>3</v>
       </c>
@@ -45245,7 +45246,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="398" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="398" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B398" s="30">
         <v>3</v>
       </c>
@@ -45332,7 +45333,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="399" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="399" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B399" s="30">
         <v>3</v>
       </c>
@@ -45418,7 +45419,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="400" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="400" spans="2:54" s="20" customFormat="1" ht="13.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B400" s="15">
         <v>2</v>
       </c>
@@ -45613,7 +45614,7 @@
         <v>0.99999999999999978</v>
       </c>
     </row>
-    <row r="401" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="401" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B401" s="30">
         <v>3</v>
       </c>
@@ -45702,7 +45703,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="402" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="402" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B402" s="30">
         <v>3</v>
       </c>
@@ -45791,7 +45792,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="403" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="403" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B403" s="30">
         <v>3</v>
       </c>
@@ -45905,7 +45906,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="404" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="404" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B404" s="30">
         <v>3</v>
       </c>
@@ -45992,7 +45993,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="405" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="405" spans="2:54" s="33" customFormat="1" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B405" s="30">
         <v>3</v>
       </c>
@@ -46079,7 +46080,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="406" spans="2:54" s="1" customFormat="1" ht="15" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="406" spans="2:54" s="1" customFormat="1" ht="14.4" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B406" s="7"/>
       <c r="C406" s="7"/>
       <c r="D406" s="7"/>
@@ -46133,7 +46134,7 @@
       <c r="BA406" s="9"/>
       <c r="BB406" s="7"/>
     </row>
-    <row r="407" spans="2:54" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="407" spans="2:54" s="1" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B407" s="10">
         <v>1</v>
       </c>
@@ -46331,7 +46332,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="408" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="408" spans="2:54" s="20" customFormat="1" ht="13.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B408" s="15">
         <v>2</v>
       </c>
@@ -46526,7 +46527,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="409" spans="2:54" s="36" customFormat="1" ht="13.5" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="409" spans="2:54" s="36" customFormat="1" ht="13.8" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B409" s="30">
         <v>3</v>
       </c>
@@ -46609,7 +46610,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="410" spans="2:54" s="33" customFormat="1" ht="13.5" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="410" spans="2:54" s="33" customFormat="1" ht="13.8" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B410" s="30">
         <v>3</v>
       </c>
@@ -46692,7 +46693,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="411" spans="2:54" s="33" customFormat="1" ht="13.5" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="411" spans="2:54" s="33" customFormat="1" ht="13.8" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B411" s="30">
         <v>3</v>
       </c>
@@ -46775,7 +46776,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="412" spans="2:54" s="33" customFormat="1" ht="13.5" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="412" spans="2:54" s="33" customFormat="1" ht="13.8" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B412" s="30">
         <v>3</v>
       </c>
@@ -46858,7 +46859,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="413" spans="2:54" s="33" customFormat="1" ht="13.5" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="413" spans="2:54" s="33" customFormat="1" ht="13.8" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B413" s="30">
         <v>3</v>
       </c>
@@ -46941,7 +46942,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="414" spans="2:54" s="33" customFormat="1" ht="13.5" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="414" spans="2:54" s="33" customFormat="1" ht="13.8" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B414" s="30">
         <v>3</v>
       </c>
@@ -47024,7 +47025,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="415" spans="2:54" s="33" customFormat="1" ht="13.5" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="415" spans="2:54" s="33" customFormat="1" ht="13.8" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B415" s="30">
         <v>3</v>
       </c>
@@ -47107,7 +47108,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="416" spans="2:54" s="33" customFormat="1" ht="13.5" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="416" spans="2:54" s="33" customFormat="1" ht="13.8" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B416" s="30">
         <v>3</v>
       </c>
@@ -47190,7 +47191,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="417" spans="2:54" s="33" customFormat="1" ht="13.5" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="417" spans="2:54" s="33" customFormat="1" ht="13.8" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B417" s="30">
         <v>3</v>
       </c>
@@ -47273,7 +47274,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="418" spans="2:54" s="36" customFormat="1" ht="13.5" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="418" spans="2:54" s="36" customFormat="1" ht="13.8" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B418" s="30">
         <v>3</v>
       </c>
@@ -47356,7 +47357,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="419" spans="2:54" s="33" customFormat="1" ht="13.5" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="419" spans="2:54" s="33" customFormat="1" ht="13.8" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B419" s="30">
         <v>3</v>
       </c>
@@ -47439,7 +47440,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="420" spans="2:54" s="33" customFormat="1" ht="13.5" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="420" spans="2:54" s="33" customFormat="1" ht="13.8" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B420" s="30">
         <v>3</v>
       </c>
@@ -47522,7 +47523,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="421" spans="2:54" s="33" customFormat="1" ht="13.5" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="421" spans="2:54" s="33" customFormat="1" ht="13.8" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B421" s="30">
         <v>3</v>
       </c>
@@ -47605,7 +47606,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="422" spans="2:54" s="33" customFormat="1" ht="13.5" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="422" spans="2:54" s="33" customFormat="1" ht="13.8" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B422" s="30">
         <v>3</v>
       </c>
@@ -47720,7 +47721,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="423" spans="2:54" s="1" customFormat="1" ht="15" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="423" spans="2:54" s="1" customFormat="1" ht="14.4" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B423" s="7"/>
       <c r="C423" s="7"/>
       <c r="D423" s="7"/>
@@ -47774,7 +47775,7 @@
       <c r="BA423" s="9"/>
       <c r="BB423" s="9"/>
     </row>
-    <row r="424" spans="2:54" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+    <row r="424" spans="2:54" s="1" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B424" s="10">
         <v>1</v>
       </c>
@@ -47972,7 +47973,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="425" spans="2:54" s="20" customFormat="1" ht="13.5" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="425" spans="2:54" s="20" customFormat="1" ht="13.8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="B425" s="15">
         <v>2</v>
       </c>
@@ -48173,7 +48174,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="426" spans="2:54" s="36" customFormat="1" ht="13.5" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="426" spans="2:54" s="36" customFormat="1" ht="13.8" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B426" s="30">
         <v>3</v>
       </c>
@@ -48360,7 +48361,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="427" spans="2:54" s="33" customFormat="1" ht="13.5" outlineLevel="2" x14ac:dyDescent="0.25">
+    <row r="427" spans="2:54" s="33" customFormat="1" ht="13.8" outlineLevel="2" x14ac:dyDescent="0.3">
       <c r="B427" s="30">
         <v>3</v>
       </c>
@@ -48726,293 +48727,294 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59A9A9A2-AF59-4E23-8473-E3235F07F470}">
+  <sheetPr codeName="Planilha2"/>
   <dimension ref="A1:A57"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A57" s="1"/>
     </row>
   </sheetData>
@@ -49033,15 +49035,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100DBAF84C653C70648848D5CE3F55E0766" ma:contentTypeVersion="15" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="c32e246f0697ea5fff0ff7310475e255">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="fd7a431a-ac48-40c9-8cfb-fb570019eb11" xmlns:ns3="c220fbd3-771c-45fb-b226-1e7078e429df" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f2dffe092b16b70d30aebcfa0a94d9c9" ns2:_="" ns3:_="">
     <xsd:import namespace="fd7a431a-ac48-40c9-8cfb-fb570019eb11"/>
@@ -49276,6 +49269,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2F5B731-90EB-4058-9385-4A87D458D64A}">
   <ds:schemaRefs>
@@ -49288,14 +49290,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5EB9E8F0-F327-4E84-B990-6EC8B9560054}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B10762B-3A52-4D91-AC69-FE0CB85E07A4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -49312,4 +49306,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5EB9E8F0-F327-4E84-B990-6EC8B9560054}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
fix(orcamento): codigos 16.2.x duplicados — renomeia para 16.3.x na tarefa 16.3 EQUIPAMENTOS SDAI (migration 047)
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Cronograma Físico Financeiro WAVE - FIP rev 07 percentuais.xlsx
+++ b/docs/Cronograma Físico Financeiro WAVE - FIP rev 07 percentuais.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b73f7ac4adb68b79/APP-GESTAO-CONTRATO/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="550" documentId="8_{66E8BC8A-DCAE-49C6-B59C-AFC9CA3C8614}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3BED2328-E662-482B-885B-EF08A09B2C7A}"/>
+  <xr:revisionPtr revIDLastSave="552" documentId="8_{66E8BC8A-DCAE-49C6-B59C-AFC9CA3C8614}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8E25E4E1-C51D-4BA8-B604-B0D57D4CDF89}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="601" xr2:uid="{37B66749-6C7B-43A5-9069-298DC434CDF1}"/>
+    <workbookView minimized="1" xWindow="5952" yWindow="4008" windowWidth="17280" windowHeight="8928" tabRatio="601" xr2:uid="{37B66749-6C7B-43A5-9069-298DC434CDF1}"/>
   </bookViews>
   <sheets>
     <sheet name="serviço" sheetId="1" r:id="rId1"/>
@@ -99,7 +99,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1651" uniqueCount="812">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1651" uniqueCount="826">
   <si>
     <t>DISCIPLINA</t>
   </si>
@@ -2565,6 +2565,48 @@
   </si>
   <si>
     <t>ACUMULADO</t>
+  </si>
+  <si>
+    <t>16,.3.1</t>
+  </si>
+  <si>
+    <t>16,.3.2</t>
+  </si>
+  <si>
+    <t>16,.3.3</t>
+  </si>
+  <si>
+    <t>16,.3.4</t>
+  </si>
+  <si>
+    <t>16,.3.5</t>
+  </si>
+  <si>
+    <t>16,.3.6</t>
+  </si>
+  <si>
+    <t>16,.3.7</t>
+  </si>
+  <si>
+    <t>16,.3.8</t>
+  </si>
+  <si>
+    <t>16,.3.9</t>
+  </si>
+  <si>
+    <t>16,.3.10</t>
+  </si>
+  <si>
+    <t>16,.3.11</t>
+  </si>
+  <si>
+    <t>16,.3.12</t>
+  </si>
+  <si>
+    <t>16,.3.13</t>
+  </si>
+  <si>
+    <t>16,.3.14</t>
   </si>
 </sst>
 </file>
@@ -43154,7 +43196,7 @@
         <v>601</v>
       </c>
       <c r="D377" s="30" t="s">
-        <v>237</v>
+        <v>812</v>
       </c>
       <c r="E377" s="37" t="s">
         <v>641</v>
@@ -43241,7 +43283,7 @@
         <v>601</v>
       </c>
       <c r="D378" s="30" t="s">
-        <v>238</v>
+        <v>813</v>
       </c>
       <c r="E378" s="37" t="s">
         <v>642</v>
@@ -43328,7 +43370,7 @@
         <v>601</v>
       </c>
       <c r="D379" s="30" t="s">
-        <v>239</v>
+        <v>814</v>
       </c>
       <c r="E379" s="37" t="s">
         <v>643</v>
@@ -43415,7 +43457,7 @@
         <v>601</v>
       </c>
       <c r="D380" s="30" t="s">
-        <v>240</v>
+        <v>815</v>
       </c>
       <c r="E380" s="37" t="s">
         <v>644</v>
@@ -43502,7 +43544,7 @@
         <v>601</v>
       </c>
       <c r="D381" s="30" t="s">
-        <v>241</v>
+        <v>816</v>
       </c>
       <c r="E381" s="37" t="s">
         <v>645</v>
@@ -43589,7 +43631,7 @@
         <v>601</v>
       </c>
       <c r="D382" s="30" t="s">
-        <v>242</v>
+        <v>817</v>
       </c>
       <c r="E382" s="37" t="s">
         <v>646</v>
@@ -43676,7 +43718,7 @@
         <v>601</v>
       </c>
       <c r="D383" s="30" t="s">
-        <v>243</v>
+        <v>818</v>
       </c>
       <c r="E383" s="37" t="s">
         <v>647</v>
@@ -43763,7 +43805,7 @@
         <v>601</v>
       </c>
       <c r="D384" s="30" t="s">
-        <v>244</v>
+        <v>819</v>
       </c>
       <c r="E384" s="37" t="s">
         <v>648</v>
@@ -43850,7 +43892,7 @@
         <v>601</v>
       </c>
       <c r="D385" s="30" t="s">
-        <v>602</v>
+        <v>820</v>
       </c>
       <c r="E385" s="37" t="s">
         <v>649</v>
@@ -43937,7 +43979,7 @@
         <v>601</v>
       </c>
       <c r="D386" s="30" t="s">
-        <v>603</v>
+        <v>821</v>
       </c>
       <c r="E386" s="37" t="s">
         <v>650</v>
@@ -44024,7 +44066,7 @@
         <v>601</v>
       </c>
       <c r="D387" s="30" t="s">
-        <v>604</v>
+        <v>822</v>
       </c>
       <c r="E387" s="37" t="s">
         <v>651</v>
@@ -44116,7 +44158,7 @@
         <v>601</v>
       </c>
       <c r="D388" s="30" t="s">
-        <v>605</v>
+        <v>823</v>
       </c>
       <c r="E388" s="37" t="s">
         <v>652</v>
@@ -44203,7 +44245,7 @@
         <v>601</v>
       </c>
       <c r="D389" s="30" t="s">
-        <v>606</v>
+        <v>824</v>
       </c>
       <c r="E389" s="37" t="s">
         <v>653</v>
@@ -44291,7 +44333,7 @@
         <v>601</v>
       </c>
       <c r="D390" s="30" t="s">
-        <v>607</v>
+        <v>825</v>
       </c>
       <c r="E390" s="37" t="s">
         <v>654</v>
@@ -49021,26 +49063,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="fd7a431a-ac48-40c9-8cfb-fb570019eb11" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c220fbd3-771c-45fb-b226-1e7078e429df">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100DBAF84C653C70648848D5CE3F55E0766" ma:contentTypeVersion="15" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="c32e246f0697ea5fff0ff7310475e255">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="fd7a431a-ac48-40c9-8cfb-fb570019eb11" xmlns:ns3="c220fbd3-771c-45fb-b226-1e7078e429df" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f2dffe092b16b70d30aebcfa0a94d9c9" ns2:_="" ns3:_="">
     <xsd:import namespace="fd7a431a-ac48-40c9-8cfb-fb570019eb11"/>
@@ -49275,26 +49297,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2F5B731-90EB-4058-9385-4A87D458D64A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="fd7a431a-ac48-40c9-8cfb-fb570019eb11"/>
-    <ds:schemaRef ds:uri="c220fbd3-771c-45fb-b226-1e7078e429df"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5EB9E8F0-F327-4E84-B990-6EC8B9560054}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="fd7a431a-ac48-40c9-8cfb-fb570019eb11" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c220fbd3-771c-45fb-b226-1e7078e429df">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B10762B-3A52-4D91-AC69-FE0CB85E07A4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -49311,4 +49334,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5EB9E8F0-F327-4E84-B990-6EC8B9560054}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2F5B731-90EB-4058-9385-4A87D458D64A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="fd7a431a-ac48-40c9-8cfb-fb570019eb11"/>
+    <ds:schemaRef ds:uri="c220fbd3-771c-45fb-b226-1e7078e429df"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat(orcamento): template xlsx 8 colunas + upload para reajuste em massa
Fluxo novo na aba Estrutura do contrato:
- 'Baixar planilha' → GET /api/contratos/[id]/orcamento/template
  Entrega xlsx no formato da planilha oficial (8 colunas):
  Cód / Descrição / Local / Qtde / Unid / PR. Mat / PR. M.O. / Total
  Coluna técnica detalhamento_id fica oculta ao lado.
  Ordenação natural por código (1.2 < 1.10 < 2.1).
- 'Subir planilha' → POST /api/contratos/[id]/orcamento/upload
  Lê a aba Orcamento e atualiza Qtde, PR. Mat e PR. M.O. nos dets
  pelo detalhamento_id (ou fallback por Cód.). Recalcula valor_unitario
  e valor_total. Só atualiza linhas nível 3 (ignora headers de grupo/tarefa).

Uso típico: baixar → aplicar +10% via 'Colar especial → Multiplicar' no Excel → subir.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Cronograma Físico Financeiro WAVE - FIP rev 07 percentuais.xlsx
+++ b/docs/Cronograma Físico Financeiro WAVE - FIP rev 07 percentuais.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b73f7ac4adb68b79/APP-GESTAO-CONTRATO/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="552" documentId="8_{66E8BC8A-DCAE-49C6-B59C-AFC9CA3C8614}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8E25E4E1-C51D-4BA8-B604-B0D57D4CDF89}"/>
+  <xr:revisionPtr revIDLastSave="565" documentId="8_{66E8BC8A-DCAE-49C6-B59C-AFC9CA3C8614}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BBC88EDA-F4C4-4A83-9B15-430731254D00}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="5952" yWindow="4008" windowWidth="17280" windowHeight="8928" tabRatio="601" xr2:uid="{37B66749-6C7B-43A5-9069-298DC434CDF1}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="601" xr2:uid="{37B66749-6C7B-43A5-9069-298DC434CDF1}"/>
   </bookViews>
   <sheets>
     <sheet name="serviço" sheetId="1" r:id="rId1"/>
@@ -99,7 +99,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1651" uniqueCount="826">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1651" uniqueCount="846">
   <si>
     <t>DISCIPLINA</t>
   </si>
@@ -1808,9 +1808,6 @@
   </si>
   <si>
     <t>15.1.14</t>
-  </si>
-  <si>
-    <t>15.1.15</t>
   </si>
   <si>
     <t>INCENDIO</t>
@@ -2567,46 +2564,109 @@
     <t>ACUMULADO</t>
   </si>
   <si>
-    <t>16,.3.1</t>
-  </si>
-  <si>
-    <t>16,.3.2</t>
-  </si>
-  <si>
-    <t>16,.3.3</t>
-  </si>
-  <si>
-    <t>16,.3.4</t>
-  </si>
-  <si>
-    <t>16,.3.5</t>
-  </si>
-  <si>
-    <t>16,.3.6</t>
-  </si>
-  <si>
-    <t>16,.3.7</t>
-  </si>
-  <si>
-    <t>16,.3.8</t>
-  </si>
-  <si>
-    <t>16,.3.9</t>
-  </si>
-  <si>
-    <t>16,.3.10</t>
-  </si>
-  <si>
-    <t>16,.3.11</t>
-  </si>
-  <si>
-    <t>16,.3.12</t>
-  </si>
-  <si>
-    <t>16,.3.13</t>
-  </si>
-  <si>
-    <t>16,.3.14</t>
+    <t>15.2.1</t>
+  </si>
+  <si>
+    <t>15.2.2</t>
+  </si>
+  <si>
+    <t>15.2.3</t>
+  </si>
+  <si>
+    <t>15.2.4</t>
+  </si>
+  <si>
+    <t>15.2.5</t>
+  </si>
+  <si>
+    <t>15.2.6</t>
+  </si>
+  <si>
+    <t>15.2.7</t>
+  </si>
+  <si>
+    <t>15.2.8</t>
+  </si>
+  <si>
+    <t>15.2.9</t>
+  </si>
+  <si>
+    <t>15.2.10</t>
+  </si>
+  <si>
+    <t>15.2.11</t>
+  </si>
+  <si>
+    <t>15.2.12</t>
+  </si>
+  <si>
+    <t>15.2.13</t>
+  </si>
+  <si>
+    <t>15.2.14</t>
+  </si>
+  <si>
+    <t>15.2.15</t>
+  </si>
+  <si>
+    <t>16.3.1</t>
+  </si>
+  <si>
+    <t>16.3.2</t>
+  </si>
+  <si>
+    <t>16.3.3</t>
+  </si>
+  <si>
+    <t>16.3.4</t>
+  </si>
+  <si>
+    <t>16.3.5</t>
+  </si>
+  <si>
+    <t>16.3.6</t>
+  </si>
+  <si>
+    <t>16.3.7</t>
+  </si>
+  <si>
+    <t>16.3.8</t>
+  </si>
+  <si>
+    <t>16.3.9</t>
+  </si>
+  <si>
+    <t>16.3.10</t>
+  </si>
+  <si>
+    <t>16.3.11</t>
+  </si>
+  <si>
+    <t>16.3.12</t>
+  </si>
+  <si>
+    <t>16.3.13</t>
+  </si>
+  <si>
+    <t>16.3.14</t>
+  </si>
+  <si>
+    <t>17.2</t>
+  </si>
+  <si>
+    <t>17.2.1</t>
+  </si>
+  <si>
+    <t>17.2.2</t>
+  </si>
+  <si>
+    <t>17.2.3</t>
+  </si>
+  <si>
+    <t>17.2.4</t>
+  </si>
+  <si>
+    <t>17.2.5</t>
   </si>
 </sst>
 </file>
@@ -3975,7 +4035,7 @@
         <v>92</v>
       </c>
       <c r="E2" s="93" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="F2" s="90" t="s">
         <v>1</v>
@@ -4016,7 +4076,7 @@
       <c r="AE2" s="88"/>
       <c r="AF2" s="89"/>
       <c r="AH2" s="81" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="AI2" s="81"/>
       <c r="AJ2" s="81"/>
@@ -4369,7 +4429,7 @@
       <c r="C5" s="92"/>
       <c r="D5" s="85"/>
       <c r="E5" s="76" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="F5" s="92"/>
       <c r="G5" s="92"/>
@@ -5051,7 +5111,7 @@
         <v>3</v>
       </c>
       <c r="D9" s="30" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="E9" s="37" t="s">
         <v>267</v>
@@ -5327,7 +5387,7 @@
         <v>3</v>
       </c>
       <c r="D11" s="30" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="E11" s="37" t="s">
         <v>270</v>
@@ -5603,7 +5663,7 @@
         <v>3</v>
       </c>
       <c r="D13" s="30" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="E13" s="37" t="s">
         <v>268</v>
@@ -5879,7 +5939,7 @@
         <v>3</v>
       </c>
       <c r="D15" s="30" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="E15" s="37" t="s">
         <v>287</v>
@@ -6155,7 +6215,7 @@
         <v>3</v>
       </c>
       <c r="D17" s="30" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="E17" s="37" t="s">
         <v>269</v>
@@ -6240,7 +6300,7 @@
         <v>3</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="E18" s="50" t="s">
         <v>271</v>
@@ -6431,7 +6491,7 @@
         <v>3</v>
       </c>
       <c r="D19" s="30" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="E19" s="37" t="s">
         <v>271</v>
@@ -6705,7 +6765,7 @@
         <v>3</v>
       </c>
       <c r="D21" s="30" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="E21" s="37" t="s">
         <v>272</v>
@@ -6981,7 +7041,7 @@
         <v>3</v>
       </c>
       <c r="D23" s="30" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="E23" s="37" t="s">
         <v>290</v>
@@ -7255,7 +7315,7 @@
         <v>3</v>
       </c>
       <c r="D25" s="30" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="E25" s="37" t="s">
         <v>273</v>
@@ -7529,7 +7589,7 @@
         <v>3</v>
       </c>
       <c r="D27" s="30" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="E27" s="37" t="s">
         <v>274</v>
@@ -7805,7 +7865,7 @@
         <v>3</v>
       </c>
       <c r="D29" s="30" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="E29" s="37" t="s">
         <v>275</v>
@@ -8079,7 +8139,7 @@
         <v>3</v>
       </c>
       <c r="D31" s="30" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="E31" s="37" t="s">
         <v>276</v>
@@ -8353,7 +8413,7 @@
         <v>3</v>
       </c>
       <c r="D33" s="30" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="E33" s="37" t="s">
         <v>289</v>
@@ -8627,7 +8687,7 @@
         <v>3</v>
       </c>
       <c r="D35" s="30" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="E35" s="37" t="s">
         <v>288</v>
@@ -9151,7 +9211,7 @@
         <v>3</v>
       </c>
       <c r="D39" s="30" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="E39" s="37" t="s">
         <v>291</v>
@@ -9428,7 +9488,7 @@
         <v>3</v>
       </c>
       <c r="D41" s="30" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="E41" s="37" t="s">
         <v>292</v>
@@ -9705,7 +9765,7 @@
         <v>3</v>
       </c>
       <c r="D43" s="30" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="E43" s="37" t="s">
         <v>293</v>
@@ -9982,7 +10042,7 @@
         <v>3</v>
       </c>
       <c r="D45" s="30" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="E45" s="37" t="s">
         <v>294</v>
@@ -10257,7 +10317,7 @@
         <v>3</v>
       </c>
       <c r="D47" s="30" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="E47" s="37" t="s">
         <v>295</v>
@@ -10532,7 +10592,7 @@
         <v>3</v>
       </c>
       <c r="D49" s="30" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="E49" s="37" t="s">
         <v>298</v>
@@ -10807,7 +10867,7 @@
         <v>3</v>
       </c>
       <c r="D51" s="30" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="E51" s="37" t="s">
         <v>296</v>
@@ -11086,7 +11146,7 @@
         <v>3</v>
       </c>
       <c r="D53" s="30" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="E53" s="37" t="s">
         <v>297</v>
@@ -11363,7 +11423,7 @@
         <v>3</v>
       </c>
       <c r="D55" s="30" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="E55" s="37" t="s">
         <v>299</v>
@@ -13084,10 +13144,10 @@
         <v>323</v>
       </c>
       <c r="E73" s="37" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="F73" s="31" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="G73" s="30">
         <v>50</v>
@@ -18001,7 +18061,7 @@
         <v>394</v>
       </c>
       <c r="E124" s="37" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="F124" s="31" t="s">
         <v>8</v>
@@ -18093,7 +18153,7 @@
         <v>395</v>
       </c>
       <c r="E125" s="37" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="F125" s="31" t="s">
         <v>9</v>
@@ -18184,7 +18244,7 @@
         <v>396</v>
       </c>
       <c r="E126" s="37" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="F126" s="31" t="s">
         <v>10</v>
@@ -18275,7 +18335,7 @@
         <v>397</v>
       </c>
       <c r="E127" s="37" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="F127" s="31" t="s">
         <v>11</v>
@@ -18366,7 +18426,7 @@
         <v>398</v>
       </c>
       <c r="E128" s="37" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="F128" s="31" t="s">
         <v>12</v>
@@ -18457,7 +18517,7 @@
         <v>399</v>
       </c>
       <c r="E129" s="37" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="F129" s="31" t="s">
         <v>13</v>
@@ -18548,7 +18608,7 @@
         <v>400</v>
       </c>
       <c r="E130" s="37" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="F130" s="31" t="s">
         <v>14</v>
@@ -18639,7 +18699,7 @@
         <v>401</v>
       </c>
       <c r="E131" s="37" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="F131" s="31" t="s">
         <v>15</v>
@@ -18730,7 +18790,7 @@
         <v>402</v>
       </c>
       <c r="E132" s="37" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="F132" s="31" t="s">
         <v>17</v>
@@ -18821,7 +18881,7 @@
         <v>403</v>
       </c>
       <c r="E133" s="37" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="F133" s="31" t="s">
         <v>16</v>
@@ -18912,7 +18972,7 @@
         <v>404</v>
       </c>
       <c r="E134" s="37" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="F134" s="31" t="s">
         <v>91</v>
@@ -19002,7 +19062,7 @@
         <v>405</v>
       </c>
       <c r="E135" s="37" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="F135" s="31" t="s">
         <v>55</v>
@@ -19093,7 +19153,7 @@
         <v>406</v>
       </c>
       <c r="E136" s="37" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="F136" s="31" t="s">
         <v>56</v>
@@ -19184,7 +19244,7 @@
         <v>407</v>
       </c>
       <c r="E137" s="37" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="F137" s="31" t="s">
         <v>58</v>
@@ -19525,7 +19585,7 @@
         <v>127</v>
       </c>
       <c r="E140" s="50" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="F140" s="15" t="s">
         <v>60</v>
@@ -19725,7 +19785,7 @@
         <v>128</v>
       </c>
       <c r="E141" s="37" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="F141" s="31" t="s">
         <v>8</v>
@@ -19971,7 +20031,7 @@
         <v>131</v>
       </c>
       <c r="E144" s="37" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="F144" s="31" t="s">
         <v>11</v>
@@ -20299,7 +20359,7 @@
         <v>135</v>
       </c>
       <c r="E148" s="37" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="F148" s="31" t="s">
         <v>15</v>
@@ -20467,7 +20527,7 @@
         <v>420</v>
       </c>
       <c r="E150" s="37" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="F150" s="31" t="s">
         <v>16</v>
@@ -21245,7 +21305,7 @@
         <v>138</v>
       </c>
       <c r="E158" s="51" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="F158" s="15" t="s">
         <v>60</v>
@@ -21446,7 +21506,7 @@
         <v>139</v>
       </c>
       <c r="E159" s="37" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="F159" s="31" t="s">
         <v>8</v>
@@ -21529,7 +21589,7 @@
         <v>140</v>
       </c>
       <c r="E160" s="37" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="F160" s="31" t="s">
         <v>9</v>
@@ -21612,7 +21672,7 @@
         <v>141</v>
       </c>
       <c r="E161" s="37" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="F161" s="31" t="s">
         <v>10</v>
@@ -21695,7 +21755,7 @@
         <v>142</v>
       </c>
       <c r="E162" s="37" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="F162" s="31" t="s">
         <v>11</v>
@@ -21778,7 +21838,7 @@
         <v>143</v>
       </c>
       <c r="E163" s="37" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="F163" s="31" t="s">
         <v>12</v>
@@ -21861,7 +21921,7 @@
         <v>144</v>
       </c>
       <c r="E164" s="37" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="F164" s="31" t="s">
         <v>13</v>
@@ -21944,7 +22004,7 @@
         <v>145</v>
       </c>
       <c r="E165" s="37" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="F165" s="31" t="s">
         <v>14</v>
@@ -22027,7 +22087,7 @@
         <v>146</v>
       </c>
       <c r="E166" s="37" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="F166" s="31" t="s">
         <v>15</v>
@@ -22107,10 +22167,10 @@
         <v>3</v>
       </c>
       <c r="D167" s="30" t="s">
+        <v>581</v>
+      </c>
+      <c r="E167" s="37" t="s">
         <v>582</v>
-      </c>
-      <c r="E167" s="37" t="s">
-        <v>583</v>
       </c>
       <c r="F167" s="31" t="s">
         <v>17</v>
@@ -22190,10 +22250,10 @@
         <v>3</v>
       </c>
       <c r="D168" s="30" t="s">
+        <v>583</v>
+      </c>
+      <c r="E168" s="37" t="s">
         <v>584</v>
-      </c>
-      <c r="E168" s="37" t="s">
-        <v>585</v>
       </c>
       <c r="F168" s="31" t="s">
         <v>16</v>
@@ -22273,10 +22333,10 @@
         <v>3</v>
       </c>
       <c r="D169" s="30" t="s">
+        <v>585</v>
+      </c>
+      <c r="E169" s="37" t="s">
         <v>586</v>
-      </c>
-      <c r="E169" s="37" t="s">
-        <v>587</v>
       </c>
       <c r="F169" s="31" t="s">
         <v>91</v>
@@ -22377,10 +22437,10 @@
         <v>3</v>
       </c>
       <c r="D170" s="30" t="s">
+        <v>587</v>
+      </c>
+      <c r="E170" s="37" t="s">
         <v>588</v>
-      </c>
-      <c r="E170" s="37" t="s">
-        <v>589</v>
       </c>
       <c r="F170" s="31" t="s">
         <v>55</v>
@@ -22462,10 +22522,10 @@
         <v>3</v>
       </c>
       <c r="D171" s="30" t="s">
+        <v>589</v>
+      </c>
+      <c r="E171" s="37" t="s">
         <v>590</v>
-      </c>
-      <c r="E171" s="37" t="s">
-        <v>591</v>
       </c>
       <c r="F171" s="31" t="s">
         <v>56</v>
@@ -22547,10 +22607,10 @@
         <v>3</v>
       </c>
       <c r="D172" s="30" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="E172" s="37" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="F172" s="31" t="s">
         <v>58</v>
@@ -24351,7 +24411,7 @@
         <v>157</v>
       </c>
       <c r="E190" s="51" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="F190" s="15" t="s">
         <v>60</v>
@@ -24546,10 +24606,10 @@
         <v>158</v>
       </c>
       <c r="E191" s="37" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="F191" s="31" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="G191" s="30">
         <v>48</v>
@@ -24656,7 +24716,7 @@
         <v>159</v>
       </c>
       <c r="E192" s="70" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="F192" s="31" t="s">
         <v>8</v>
@@ -24739,7 +24799,7 @@
         <v>160</v>
       </c>
       <c r="E193" s="70" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="F193" s="31" t="s">
         <v>9</v>
@@ -24822,7 +24882,7 @@
         <v>161</v>
       </c>
       <c r="E194" s="70" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="F194" s="31" t="s">
         <v>10</v>
@@ -24905,7 +24965,7 @@
         <v>162</v>
       </c>
       <c r="E195" s="37" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="F195" s="31" t="s">
         <v>11</v>
@@ -25765,7 +25825,7 @@
         <v>4</v>
       </c>
       <c r="D205" s="30" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="E205" s="37" t="s">
         <v>459</v>
@@ -25848,7 +25908,7 @@
         <v>4</v>
       </c>
       <c r="D206" s="30" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="E206" s="37" t="s">
         <v>460</v>
@@ -25931,7 +25991,7 @@
         <v>4</v>
       </c>
       <c r="D207" s="30" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="E207" s="37" t="s">
         <v>461</v>
@@ -26212,7 +26272,7 @@
         <v>167</v>
       </c>
       <c r="E209" s="37" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="F209" s="37" t="s">
         <v>60</v>
@@ -26545,7 +26605,7 @@
         <v>168</v>
       </c>
       <c r="E212" s="51" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="F212" s="15" t="s">
         <v>60</v>
@@ -26740,10 +26800,10 @@
         <v>169</v>
       </c>
       <c r="E213" s="37" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="F213" s="31" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="G213" s="30">
         <v>48</v>
@@ -28585,10 +28645,10 @@
         <v>178</v>
       </c>
       <c r="E232" s="37" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="F232" s="31" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="G232" s="30">
         <v>48</v>
@@ -28695,7 +28755,7 @@
         <v>179</v>
       </c>
       <c r="E233" s="37" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="F233" s="31" t="s">
         <v>8</v>
@@ -28778,7 +28838,7 @@
         <v>180</v>
       </c>
       <c r="E234" s="37" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="F234" s="31" t="s">
         <v>9</v>
@@ -28861,7 +28921,7 @@
         <v>181</v>
       </c>
       <c r="E235" s="37" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="F235" s="31" t="s">
         <v>10</v>
@@ -28944,7 +29004,7 @@
         <v>182</v>
       </c>
       <c r="E236" s="37" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="F236" s="31" t="s">
         <v>11</v>
@@ -29027,7 +29087,7 @@
         <v>183</v>
       </c>
       <c r="E237" s="37" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="F237" s="31" t="s">
         <v>12</v>
@@ -29112,7 +29172,7 @@
         <v>184</v>
       </c>
       <c r="E238" s="37" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="F238" s="31" t="s">
         <v>13</v>
@@ -29185,7 +29245,7 @@
         <v>185</v>
       </c>
       <c r="E239" s="37" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="F239" s="31" t="s">
         <v>14</v>
@@ -29270,7 +29330,7 @@
         <v>503</v>
       </c>
       <c r="E240" s="37" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="F240" s="31" t="s">
         <v>14</v>
@@ -29353,7 +29413,7 @@
         <v>504</v>
       </c>
       <c r="E241" s="37" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="F241" s="31" t="s">
         <v>17</v>
@@ -29438,7 +29498,7 @@
         <v>505</v>
       </c>
       <c r="E242" s="37" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="F242" s="31" t="s">
         <v>16</v>
@@ -29523,7 +29583,7 @@
         <v>506</v>
       </c>
       <c r="E243" s="37" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="F243" s="31" t="s">
         <v>91</v>
@@ -29635,7 +29695,7 @@
         <v>507</v>
       </c>
       <c r="E244" s="37" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="F244" s="31" t="s">
         <v>55</v>
@@ -29720,7 +29780,7 @@
         <v>508</v>
       </c>
       <c r="E245" s="37" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="F245" s="31" t="s">
         <v>56</v>
@@ -29802,10 +29862,10 @@
         <v>502</v>
       </c>
       <c r="D246" s="30" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E246" s="37" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="F246" s="31" t="s">
         <v>58</v>
@@ -31006,7 +31066,7 @@
         <v>196</v>
       </c>
       <c r="E257" s="52" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="F257" s="38" t="s">
         <v>60</v>
@@ -32187,7 +32247,7 @@
         <v>1</v>
       </c>
       <c r="C269" s="10" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="D269" s="10">
         <v>13</v>
@@ -32379,13 +32439,13 @@
         <v>2</v>
       </c>
       <c r="C270" s="15" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="D270" s="15" t="s">
         <v>200</v>
       </c>
       <c r="E270" s="51" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="F270" s="15" t="s">
         <v>60</v>
@@ -32573,7 +32633,7 @@
         <v>3</v>
       </c>
       <c r="C271" s="30" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="D271" s="30" t="s">
         <v>201</v>
@@ -32663,7 +32723,7 @@
         <v>3</v>
       </c>
       <c r="C272" s="30" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="D272" s="30" t="s">
         <v>202</v>
@@ -32753,7 +32813,7 @@
         <v>3</v>
       </c>
       <c r="C273" s="30" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="D273" s="30" t="s">
         <v>203</v>
@@ -32843,7 +32903,7 @@
         <v>3</v>
       </c>
       <c r="C274" s="30" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="D274" s="30" t="s">
         <v>204</v>
@@ -32929,7 +32989,7 @@
         <v>3</v>
       </c>
       <c r="C275" s="30" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="D275" s="30" t="s">
         <v>205</v>
@@ -33013,7 +33073,7 @@
         <v>2</v>
       </c>
       <c r="C276" s="15" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="D276" s="15" t="s">
         <v>206</v>
@@ -33206,7 +33266,7 @@
         <v>3</v>
       </c>
       <c r="C277" s="30" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="D277" s="30" t="s">
         <v>207</v>
@@ -33310,7 +33370,7 @@
         <v>3</v>
       </c>
       <c r="C278" s="30" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="D278" s="30" t="s">
         <v>208</v>
@@ -33840,7 +33900,7 @@
         <v>3</v>
       </c>
       <c r="C282" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D282" s="30" t="s">
         <v>210</v>
@@ -33849,7 +33909,7 @@
         <v>527</v>
       </c>
       <c r="F282" s="31" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="G282" s="30">
         <v>48</v>
@@ -33953,7 +34013,7 @@
         <v>3</v>
       </c>
       <c r="C283" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D283" s="30" t="s">
         <v>211</v>
@@ -34066,7 +34126,7 @@
         <v>3</v>
       </c>
       <c r="C284" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D284" s="30" t="s">
         <v>212</v>
@@ -34152,7 +34212,7 @@
         <v>3</v>
       </c>
       <c r="C285" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D285" s="30" t="s">
         <v>213</v>
@@ -34238,7 +34298,7 @@
         <v>3</v>
       </c>
       <c r="C286" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D286" s="30" t="s">
         <v>214</v>
@@ -34324,13 +34384,13 @@
         <v>3</v>
       </c>
       <c r="C287" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D287" s="30" t="s">
         <v>215</v>
       </c>
       <c r="E287" s="37" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="F287" s="31" t="s">
         <v>91</v>
@@ -34437,7 +34497,7 @@
         <v>3</v>
       </c>
       <c r="C288" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D288" s="30" t="s">
         <v>216</v>
@@ -34524,7 +34584,7 @@
         <v>3</v>
       </c>
       <c r="C289" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D289" s="30" t="s">
         <v>217</v>
@@ -34806,16 +34866,16 @@
         <v>3</v>
       </c>
       <c r="C291" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D291" s="30" t="s">
         <v>219</v>
       </c>
       <c r="E291" s="37" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="F291" s="31" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="G291" s="30">
         <v>48</v>
@@ -34945,7 +35005,7 @@
         <v>3</v>
       </c>
       <c r="C292" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D292" s="30" t="s">
         <v>220</v>
@@ -35032,13 +35092,13 @@
         <v>3</v>
       </c>
       <c r="C293" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D293" s="30" t="s">
         <v>221</v>
       </c>
       <c r="E293" s="37" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="F293" s="31" t="s">
         <v>8</v>
@@ -35121,13 +35181,13 @@
         <v>3</v>
       </c>
       <c r="C294" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D294" s="30" t="s">
         <v>222</v>
       </c>
       <c r="E294" s="37" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="F294" s="31" t="s">
         <v>9</v>
@@ -35210,13 +35270,13 @@
         <v>3</v>
       </c>
       <c r="C295" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D295" s="30" t="s">
         <v>223</v>
       </c>
       <c r="E295" s="37" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="F295" s="31" t="s">
         <v>10</v>
@@ -35299,13 +35359,13 @@
         <v>3</v>
       </c>
       <c r="C296" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D296" s="30" t="s">
         <v>224</v>
       </c>
       <c r="E296" s="37" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="F296" s="31" t="s">
         <v>11</v>
@@ -35388,13 +35448,13 @@
         <v>3</v>
       </c>
       <c r="C297" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D297" s="30" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="E297" s="37" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="F297" s="31" t="s">
         <v>12</v>
@@ -35476,13 +35536,13 @@
         <v>3</v>
       </c>
       <c r="C298" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D298" s="30" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="E298" s="37" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="F298" s="31" t="s">
         <v>13</v>
@@ -35565,13 +35625,13 @@
         <v>3</v>
       </c>
       <c r="C299" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D299" s="30" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="E299" s="37" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="F299" s="31" t="s">
         <v>14</v>
@@ -35654,13 +35714,13 @@
         <v>3</v>
       </c>
       <c r="C300" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D300" s="30" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="E300" s="37" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="F300" s="31" t="s">
         <v>15</v>
@@ -35743,13 +35803,13 @@
         <v>3</v>
       </c>
       <c r="C301" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D301" s="30" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="E301" s="37" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="F301" s="31" t="s">
         <v>17</v>
@@ -35830,13 +35890,13 @@
         <v>3</v>
       </c>
       <c r="C302" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D302" s="30" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="E302" s="37" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="F302" s="31" t="s">
         <v>16</v>
@@ -35919,10 +35979,10 @@
         <v>3</v>
       </c>
       <c r="C303" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D303" s="30" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="E303" s="37" t="s">
         <v>535</v>
@@ -36059,10 +36119,10 @@
         <v>3</v>
       </c>
       <c r="C304" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D304" s="30" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="E304" s="37" t="s">
         <v>536</v>
@@ -36145,10 +36205,10 @@
         <v>3</v>
       </c>
       <c r="C305" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D305" s="30" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="E305" s="37" t="s">
         <v>537</v>
@@ -36231,10 +36291,10 @@
         <v>3</v>
       </c>
       <c r="C306" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D306" s="30" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="E306" s="37" t="s">
         <v>538</v>
@@ -36317,7 +36377,7 @@
         <v>2</v>
       </c>
       <c r="C307" s="67" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D307" s="15" t="s">
         <v>225</v>
@@ -36512,7 +36572,7 @@
         <v>3</v>
       </c>
       <c r="C308" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D308" s="30" t="s">
         <v>226</v>
@@ -37050,7 +37110,7 @@
         <v>3</v>
       </c>
       <c r="C312" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D312" s="30" t="s">
         <v>555</v>
@@ -37135,7 +37195,7 @@
         <v>3</v>
       </c>
       <c r="C313" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D313" s="30" t="s">
         <v>556</v>
@@ -37220,7 +37280,7 @@
         <v>3</v>
       </c>
       <c r="C314" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D314" s="30" t="s">
         <v>557</v>
@@ -37305,7 +37365,7 @@
         <v>3</v>
       </c>
       <c r="C315" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D315" s="30" t="s">
         <v>558</v>
@@ -37390,7 +37450,7 @@
         <v>3</v>
       </c>
       <c r="C316" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D316" s="30" t="s">
         <v>559</v>
@@ -37475,7 +37535,7 @@
         <v>3</v>
       </c>
       <c r="C317" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D317" s="30" t="s">
         <v>560</v>
@@ -37560,7 +37620,7 @@
         <v>3</v>
       </c>
       <c r="C318" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D318" s="30" t="s">
         <v>561</v>
@@ -37645,7 +37705,7 @@
         <v>3</v>
       </c>
       <c r="C319" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D319" s="30" t="s">
         <v>562</v>
@@ -37730,7 +37790,7 @@
         <v>3</v>
       </c>
       <c r="C320" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D320" s="30" t="s">
         <v>563</v>
@@ -37815,7 +37875,7 @@
         <v>3</v>
       </c>
       <c r="C321" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D321" s="30" t="s">
         <v>564</v>
@@ -37900,7 +37960,7 @@
         <v>3</v>
       </c>
       <c r="C322" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D322" s="30" t="s">
         <v>565</v>
@@ -37984,7 +38044,7 @@
         <v>3</v>
       </c>
       <c r="C323" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D323" s="30" t="s">
         <v>566</v>
@@ -38069,7 +38129,7 @@
         <v>3</v>
       </c>
       <c r="C324" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D324" s="30" t="s">
         <v>567</v>
@@ -38154,7 +38214,7 @@
         <v>3</v>
       </c>
       <c r="C325" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D325" s="30" t="s">
         <v>568</v>
@@ -38242,10 +38302,10 @@
         <v>5</v>
       </c>
       <c r="D326" s="15" t="s">
+        <v>570</v>
+      </c>
+      <c r="E326" s="50" t="s">
         <v>571</v>
-      </c>
-      <c r="E326" s="50" t="s">
-        <v>572</v>
       </c>
       <c r="F326" s="15" t="s">
         <v>60</v>
@@ -38440,13 +38500,13 @@
         <v>3</v>
       </c>
       <c r="C327" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D327" s="30" t="s">
-        <v>555</v>
+        <v>811</v>
       </c>
       <c r="E327" s="37" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="F327" s="31" t="s">
         <v>8</v>
@@ -38525,13 +38585,13 @@
         <v>3</v>
       </c>
       <c r="C328" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D328" s="30" t="s">
-        <v>556</v>
+        <v>812</v>
       </c>
       <c r="E328" s="37" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="F328" s="31" t="s">
         <v>9</v>
@@ -38610,13 +38670,13 @@
         <v>3</v>
       </c>
       <c r="C329" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D329" s="30" t="s">
-        <v>557</v>
+        <v>813</v>
       </c>
       <c r="E329" s="37" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="F329" s="31" t="s">
         <v>10</v>
@@ -38695,13 +38755,13 @@
         <v>3</v>
       </c>
       <c r="C330" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D330" s="30" t="s">
-        <v>558</v>
+        <v>814</v>
       </c>
       <c r="E330" s="37" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="F330" s="31" t="s">
         <v>11</v>
@@ -38780,13 +38840,13 @@
         <v>3</v>
       </c>
       <c r="C331" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D331" s="30" t="s">
-        <v>559</v>
+        <v>815</v>
       </c>
       <c r="E331" s="37" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="F331" s="31" t="s">
         <v>12</v>
@@ -38865,13 +38925,13 @@
         <v>3</v>
       </c>
       <c r="C332" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D332" s="30" t="s">
-        <v>560</v>
+        <v>816</v>
       </c>
       <c r="E332" s="37" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="F332" s="31" t="s">
         <v>13</v>
@@ -38950,13 +39010,13 @@
         <v>3</v>
       </c>
       <c r="C333" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D333" s="30" t="s">
-        <v>561</v>
+        <v>817</v>
       </c>
       <c r="E333" s="37" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="F333" s="31" t="s">
         <v>14</v>
@@ -39035,13 +39095,13 @@
         <v>3</v>
       </c>
       <c r="C334" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D334" s="30" t="s">
-        <v>562</v>
+        <v>818</v>
       </c>
       <c r="E334" s="37" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="F334" s="31" t="s">
         <v>15</v>
@@ -39120,13 +39180,13 @@
         <v>3</v>
       </c>
       <c r="C335" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D335" s="30" t="s">
-        <v>563</v>
+        <v>819</v>
       </c>
       <c r="E335" s="37" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="F335" s="31" t="s">
         <v>17</v>
@@ -39205,13 +39265,13 @@
         <v>3</v>
       </c>
       <c r="C336" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D336" s="30" t="s">
-        <v>564</v>
+        <v>820</v>
       </c>
       <c r="E336" s="37" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="F336" s="31" t="s">
         <v>16</v>
@@ -39290,13 +39350,13 @@
         <v>3</v>
       </c>
       <c r="C337" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D337" s="30" t="s">
-        <v>565</v>
+        <v>821</v>
       </c>
       <c r="E337" s="37" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="F337" s="31" t="s">
         <v>91</v>
@@ -39376,13 +39436,13 @@
         <v>3</v>
       </c>
       <c r="C338" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D338" s="30" t="s">
-        <v>566</v>
+        <v>822</v>
       </c>
       <c r="E338" s="37" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="F338" s="31" t="s">
         <v>55</v>
@@ -39461,13 +39521,13 @@
         <v>3</v>
       </c>
       <c r="C339" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D339" s="30" t="s">
-        <v>567</v>
+        <v>823</v>
       </c>
       <c r="E339" s="37" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="F339" s="31" t="s">
         <v>56</v>
@@ -39546,13 +39606,13 @@
         <v>3</v>
       </c>
       <c r="C340" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D340" s="30" t="s">
-        <v>568</v>
+        <v>824</v>
       </c>
       <c r="E340" s="37" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="F340" s="31" t="s">
         <v>58</v>
@@ -39631,13 +39691,13 @@
         <v>3</v>
       </c>
       <c r="C341" s="30" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D341" s="30" t="s">
-        <v>569</v>
+        <v>825</v>
       </c>
       <c r="E341" s="37" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="F341" s="31" t="s">
         <v>59</v>
@@ -39769,7 +39829,7 @@
         <v>1</v>
       </c>
       <c r="C343" s="10" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D343" s="10">
         <v>16</v>
@@ -39967,13 +40027,13 @@
         <v>2</v>
       </c>
       <c r="C344" s="15" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D344" s="15" t="s">
         <v>227</v>
       </c>
       <c r="E344" s="51" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="F344" s="15" t="s">
         <v>60</v>
@@ -40167,13 +40227,13 @@
         <v>3</v>
       </c>
       <c r="C345" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D345" s="30" t="s">
         <v>228</v>
       </c>
       <c r="E345" s="37" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="F345" s="41" t="s">
         <v>8</v>
@@ -40251,13 +40311,13 @@
         <v>3</v>
       </c>
       <c r="C346" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D346" s="30" t="s">
         <v>229</v>
       </c>
       <c r="E346" s="37" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="F346" s="41" t="s">
         <v>9</v>
@@ -40335,13 +40395,13 @@
         <v>3</v>
       </c>
       <c r="C347" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D347" s="30" t="s">
         <v>230</v>
       </c>
       <c r="E347" s="37" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="F347" s="41" t="s">
         <v>10</v>
@@ -40419,13 +40479,13 @@
         <v>3</v>
       </c>
       <c r="C348" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D348" s="30" t="s">
         <v>231</v>
       </c>
       <c r="E348" s="37" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F348" s="41" t="s">
         <v>11</v>
@@ -40503,13 +40563,13 @@
         <v>3</v>
       </c>
       <c r="C349" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D349" s="30" t="s">
         <v>232</v>
       </c>
       <c r="E349" s="37" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="F349" s="41" t="s">
         <v>12</v>
@@ -40587,13 +40647,13 @@
         <v>3</v>
       </c>
       <c r="C350" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D350" s="30" t="s">
         <v>233</v>
       </c>
       <c r="E350" s="37" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="F350" s="41" t="s">
         <v>13</v>
@@ -40671,13 +40731,13 @@
         <v>3</v>
       </c>
       <c r="C351" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D351" s="30" t="s">
         <v>234</v>
       </c>
       <c r="E351" s="37" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="F351" s="41" t="s">
         <v>14</v>
@@ -40755,13 +40815,13 @@
         <v>3</v>
       </c>
       <c r="C352" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D352" s="30" t="s">
         <v>235</v>
       </c>
       <c r="E352" s="37" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="F352" s="41" t="s">
         <v>15</v>
@@ -40839,13 +40899,13 @@
         <v>3</v>
       </c>
       <c r="C353" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D353" s="30" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="E353" s="37" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="F353" s="41" t="s">
         <v>17</v>
@@ -40925,13 +40985,13 @@
         <v>3</v>
       </c>
       <c r="C354" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D354" s="30" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="E354" s="37" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="F354" s="41" t="s">
         <v>16</v>
@@ -41011,13 +41071,13 @@
         <v>3</v>
       </c>
       <c r="C355" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D355" s="30" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="E355" s="37" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="F355" s="41" t="s">
         <v>91</v>
@@ -41120,13 +41180,13 @@
         <v>3</v>
       </c>
       <c r="C356" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D356" s="30" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="E356" s="37" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="F356" s="41" t="s">
         <v>55</v>
@@ -41206,13 +41266,13 @@
         <v>3</v>
       </c>
       <c r="C357" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D357" s="30" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="E357" s="37" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="F357" s="41" t="s">
         <v>56</v>
@@ -41292,13 +41352,13 @@
         <v>3</v>
       </c>
       <c r="C358" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D358" s="30" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="E358" s="37" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="F358" s="41" t="s">
         <v>58</v>
@@ -41378,16 +41438,16 @@
         <v>3</v>
       </c>
       <c r="C359" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D359" s="30" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="E359" s="37" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="F359" s="31" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="G359" s="30">
         <v>48</v>
@@ -41489,13 +41549,13 @@
         <v>2</v>
       </c>
       <c r="C360" s="15" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D360" s="15" t="s">
         <v>236</v>
       </c>
       <c r="E360" s="51" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="F360" s="15" t="s">
         <v>60</v>
@@ -41689,13 +41749,13 @@
         <v>3</v>
       </c>
       <c r="C361" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D361" s="30" t="s">
         <v>237</v>
       </c>
       <c r="E361" s="37" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="F361" s="41" t="s">
         <v>8</v>
@@ -41772,13 +41832,13 @@
         <v>3</v>
       </c>
       <c r="C362" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D362" s="30" t="s">
         <v>238</v>
       </c>
       <c r="E362" s="37" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="F362" s="41" t="s">
         <v>9</v>
@@ -41855,13 +41915,13 @@
         <v>3</v>
       </c>
       <c r="C363" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D363" s="30" t="s">
         <v>239</v>
       </c>
       <c r="E363" s="37" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="F363" s="41" t="s">
         <v>10</v>
@@ -41938,13 +41998,13 @@
         <v>3</v>
       </c>
       <c r="C364" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D364" s="30" t="s">
         <v>240</v>
       </c>
       <c r="E364" s="37" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="F364" s="41" t="s">
         <v>11</v>
@@ -42021,13 +42081,13 @@
         <v>3</v>
       </c>
       <c r="C365" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D365" s="30" t="s">
         <v>241</v>
       </c>
       <c r="E365" s="37" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="F365" s="41" t="s">
         <v>12</v>
@@ -42104,13 +42164,13 @@
         <v>3</v>
       </c>
       <c r="C366" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D366" s="30" t="s">
         <v>242</v>
       </c>
       <c r="E366" s="37" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="F366" s="41" t="s">
         <v>13</v>
@@ -42187,13 +42247,13 @@
         <v>3</v>
       </c>
       <c r="C367" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D367" s="30" t="s">
         <v>243</v>
       </c>
       <c r="E367" s="37" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="F367" s="41" t="s">
         <v>14</v>
@@ -42270,13 +42330,13 @@
         <v>3</v>
       </c>
       <c r="C368" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D368" s="30" t="s">
         <v>244</v>
       </c>
       <c r="E368" s="37" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="F368" s="41" t="s">
         <v>15</v>
@@ -42353,13 +42413,13 @@
         <v>3</v>
       </c>
       <c r="C369" s="30" t="s">
+        <v>600</v>
+      </c>
+      <c r="D369" s="30" t="s">
         <v>601</v>
       </c>
-      <c r="D369" s="30" t="s">
-        <v>602</v>
-      </c>
       <c r="E369" s="37" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="F369" s="41" t="s">
         <v>17</v>
@@ -42438,13 +42498,13 @@
         <v>3</v>
       </c>
       <c r="C370" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D370" s="30" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="E370" s="37" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="F370" s="41" t="s">
         <v>16</v>
@@ -42521,13 +42581,13 @@
         <v>3</v>
       </c>
       <c r="C371" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D371" s="30" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="E371" s="37" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="F371" s="41" t="s">
         <v>91</v>
@@ -42631,13 +42691,13 @@
         <v>3</v>
       </c>
       <c r="C372" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D372" s="30" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="E372" s="37" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="F372" s="41" t="s">
         <v>55</v>
@@ -42716,13 +42776,13 @@
         <v>3</v>
       </c>
       <c r="C373" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D373" s="30" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="E373" s="37" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="F373" s="41" t="s">
         <v>56</v>
@@ -42801,13 +42861,13 @@
         <v>3</v>
       </c>
       <c r="C374" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D374" s="30" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="E374" s="37" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="F374" s="41" t="s">
         <v>58</v>
@@ -42886,16 +42946,16 @@
         <v>3</v>
       </c>
       <c r="C375" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D375" s="30" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="E375" s="37" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="F375" s="31" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="G375" s="30">
         <v>48</v>
@@ -42994,13 +43054,13 @@
         <v>2</v>
       </c>
       <c r="C376" s="15" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D376" s="15" t="s">
         <v>245</v>
       </c>
       <c r="E376" s="51" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="F376" s="15" t="s">
         <v>60</v>
@@ -43193,13 +43253,13 @@
         <v>3</v>
       </c>
       <c r="C377" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D377" s="30" t="s">
-        <v>812</v>
+        <v>826</v>
       </c>
       <c r="E377" s="37" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="F377" s="41" t="s">
         <v>8</v>
@@ -43280,13 +43340,13 @@
         <v>3</v>
       </c>
       <c r="C378" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D378" s="30" t="s">
-        <v>813</v>
+        <v>827</v>
       </c>
       <c r="E378" s="37" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="F378" s="41" t="s">
         <v>9</v>
@@ -43367,13 +43427,13 @@
         <v>3</v>
       </c>
       <c r="C379" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D379" s="30" t="s">
-        <v>814</v>
+        <v>828</v>
       </c>
       <c r="E379" s="37" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="F379" s="41" t="s">
         <v>10</v>
@@ -43454,13 +43514,13 @@
         <v>3</v>
       </c>
       <c r="C380" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D380" s="30" t="s">
-        <v>815</v>
+        <v>829</v>
       </c>
       <c r="E380" s="37" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="F380" s="41" t="s">
         <v>11</v>
@@ -43541,13 +43601,13 @@
         <v>3</v>
       </c>
       <c r="C381" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D381" s="30" t="s">
-        <v>816</v>
+        <v>830</v>
       </c>
       <c r="E381" s="37" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="F381" s="41" t="s">
         <v>12</v>
@@ -43628,13 +43688,13 @@
         <v>3</v>
       </c>
       <c r="C382" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D382" s="30" t="s">
-        <v>817</v>
+        <v>831</v>
       </c>
       <c r="E382" s="37" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="F382" s="41" t="s">
         <v>13</v>
@@ -43715,13 +43775,13 @@
         <v>3</v>
       </c>
       <c r="C383" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D383" s="30" t="s">
-        <v>818</v>
+        <v>832</v>
       </c>
       <c r="E383" s="37" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="F383" s="41" t="s">
         <v>14</v>
@@ -43802,13 +43862,13 @@
         <v>3</v>
       </c>
       <c r="C384" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D384" s="30" t="s">
-        <v>819</v>
+        <v>833</v>
       </c>
       <c r="E384" s="37" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="F384" s="41" t="s">
         <v>15</v>
@@ -43889,13 +43949,13 @@
         <v>3</v>
       </c>
       <c r="C385" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D385" s="30" t="s">
-        <v>820</v>
+        <v>834</v>
       </c>
       <c r="E385" s="37" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="F385" s="41" t="s">
         <v>17</v>
@@ -43976,13 +44036,13 @@
         <v>3</v>
       </c>
       <c r="C386" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D386" s="30" t="s">
-        <v>821</v>
+        <v>835</v>
       </c>
       <c r="E386" s="37" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="F386" s="41" t="s">
         <v>16</v>
@@ -44063,13 +44123,13 @@
         <v>3</v>
       </c>
       <c r="C387" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D387" s="30" t="s">
-        <v>822</v>
+        <v>836</v>
       </c>
       <c r="E387" s="37" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="F387" s="41" t="s">
         <v>91</v>
@@ -44155,13 +44215,13 @@
         <v>3</v>
       </c>
       <c r="C388" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D388" s="30" t="s">
-        <v>823</v>
+        <v>837</v>
       </c>
       <c r="E388" s="37" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="F388" s="41" t="s">
         <v>55</v>
@@ -44242,13 +44302,13 @@
         <v>3</v>
       </c>
       <c r="C389" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D389" s="30" t="s">
-        <v>824</v>
+        <v>838</v>
       </c>
       <c r="E389" s="37" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="F389" s="41" t="s">
         <v>56</v>
@@ -44330,13 +44390,13 @@
         <v>3</v>
       </c>
       <c r="C390" s="30" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D390" s="30" t="s">
-        <v>825</v>
+        <v>839</v>
       </c>
       <c r="E390" s="37" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="F390" s="41" t="s">
         <v>58</v>
@@ -44418,7 +44478,7 @@
         <v>1</v>
       </c>
       <c r="C391" s="10" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="D391" s="10">
         <v>17</v>
@@ -44610,13 +44670,13 @@
         <v>2</v>
       </c>
       <c r="C392" s="15" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="D392" s="15" t="s">
         <v>246</v>
       </c>
       <c r="E392" s="51" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="F392" s="15" t="s">
         <v>60</v>
@@ -44804,16 +44864,16 @@
         <v>3</v>
       </c>
       <c r="C393" s="30" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="D393" s="30" t="s">
         <v>247</v>
       </c>
       <c r="E393" s="37" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="F393" s="31" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="G393" s="30">
         <v>48</v>
@@ -44914,13 +44974,13 @@
         <v>3</v>
       </c>
       <c r="C394" s="30" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="D394" s="30" t="s">
         <v>248</v>
       </c>
       <c r="E394" s="37" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="F394" s="31" t="s">
         <v>12</v>
@@ -45000,13 +45060,13 @@
         <v>3</v>
       </c>
       <c r="C395" s="30" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="D395" s="30" t="s">
         <v>249</v>
       </c>
       <c r="E395" s="37" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="F395" s="31" t="s">
         <v>17</v>
@@ -45086,13 +45146,13 @@
         <v>3</v>
       </c>
       <c r="C396" s="30" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="D396" s="30" t="s">
         <v>250</v>
       </c>
       <c r="E396" s="37" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="F396" s="31" t="s">
         <v>16</v>
@@ -45174,13 +45234,13 @@
         <v>3</v>
       </c>
       <c r="C397" s="30" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="D397" s="30" t="s">
         <v>251</v>
       </c>
       <c r="E397" s="37" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="F397" s="31" t="s">
         <v>91</v>
@@ -45290,13 +45350,13 @@
         <v>3</v>
       </c>
       <c r="C398" s="30" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="D398" s="30" t="s">
         <v>252</v>
       </c>
       <c r="E398" s="37" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="F398" s="31" t="s">
         <v>55</v>
@@ -45377,13 +45437,13 @@
         <v>3</v>
       </c>
       <c r="C399" s="30" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="D399" s="30" t="s">
         <v>253</v>
       </c>
       <c r="E399" s="37" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="F399" s="31" t="s">
         <v>56</v>
@@ -45463,13 +45523,13 @@
         <v>2</v>
       </c>
       <c r="C400" s="15" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="D400" s="15" t="s">
-        <v>246</v>
+        <v>840</v>
       </c>
       <c r="E400" s="51" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="F400" s="15" t="s">
         <v>60</v>
@@ -45658,13 +45718,13 @@
         <v>3</v>
       </c>
       <c r="C401" s="30" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="D401" s="30" t="s">
-        <v>247</v>
+        <v>841</v>
       </c>
       <c r="E401" s="37" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="F401" s="31" t="s">
         <v>17</v>
@@ -45747,13 +45807,13 @@
         <v>3</v>
       </c>
       <c r="C402" s="30" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="D402" s="30" t="s">
-        <v>248</v>
+        <v>842</v>
       </c>
       <c r="E402" s="37" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="F402" s="31" t="s">
         <v>16</v>
@@ -45836,13 +45896,13 @@
         <v>3</v>
       </c>
       <c r="C403" s="30" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="D403" s="30" t="s">
-        <v>249</v>
+        <v>843</v>
       </c>
       <c r="E403" s="37" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
       <c r="F403" s="31" t="s">
         <v>91</v>
@@ -45950,13 +46010,13 @@
         <v>3</v>
       </c>
       <c r="C404" s="30" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="D404" s="30" t="s">
-        <v>250</v>
+        <v>844</v>
       </c>
       <c r="E404" s="37" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="F404" s="31" t="s">
         <v>55</v>
@@ -46037,13 +46097,13 @@
         <v>3</v>
       </c>
       <c r="C405" s="30" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="D405" s="30" t="s">
-        <v>251</v>
+        <v>845</v>
       </c>
       <c r="E405" s="37" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="F405" s="31" t="s">
         <v>56</v>
@@ -46178,7 +46238,7 @@
         <v>1</v>
       </c>
       <c r="C407" s="10" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="D407" s="10">
         <v>18</v>
@@ -46376,13 +46436,13 @@
         <v>2</v>
       </c>
       <c r="C408" s="15" t="s">
+        <v>675</v>
+      </c>
+      <c r="D408" s="15" t="s">
         <v>676</v>
       </c>
-      <c r="D408" s="15" t="s">
-        <v>677</v>
-      </c>
       <c r="E408" s="51" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="F408" s="15" t="s">
         <v>60</v>
@@ -46571,13 +46631,13 @@
         <v>3</v>
       </c>
       <c r="C409" s="30" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="D409" s="30" t="s">
         <v>254</v>
       </c>
       <c r="E409" s="37" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="F409" s="31" t="s">
         <v>8</v>
@@ -46654,13 +46714,13 @@
         <v>3</v>
       </c>
       <c r="C410" s="30" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="D410" s="30" t="s">
         <v>255</v>
       </c>
       <c r="E410" s="37" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="F410" s="31" t="s">
         <v>17</v>
@@ -46737,13 +46797,13 @@
         <v>3</v>
       </c>
       <c r="C411" s="30" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="D411" s="30" t="s">
         <v>256</v>
       </c>
       <c r="E411" s="37" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="F411" s="31" t="s">
         <v>54</v>
@@ -46820,13 +46880,13 @@
         <v>3</v>
       </c>
       <c r="C412" s="30" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="D412" s="30" t="s">
         <v>257</v>
       </c>
       <c r="E412" s="37" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="F412" s="31" t="s">
         <v>50</v>
@@ -46903,13 +46963,13 @@
         <v>3</v>
       </c>
       <c r="C413" s="30" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="D413" s="30" t="s">
         <v>258</v>
       </c>
       <c r="E413" s="37" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="F413" s="31" t="s">
         <v>46</v>
@@ -46986,13 +47046,13 @@
         <v>3</v>
       </c>
       <c r="C414" s="30" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="D414" s="30" t="s">
         <v>259</v>
       </c>
       <c r="E414" s="37" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="F414" s="31" t="s">
         <v>42</v>
@@ -47069,13 +47129,13 @@
         <v>3</v>
       </c>
       <c r="C415" s="30" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="D415" s="30" t="s">
         <v>260</v>
       </c>
       <c r="E415" s="37" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="F415" s="31" t="s">
         <v>38</v>
@@ -47152,13 +47212,13 @@
         <v>3</v>
       </c>
       <c r="C416" s="30" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="D416" s="30" t="s">
         <v>261</v>
       </c>
       <c r="E416" s="37" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="F416" s="31" t="s">
         <v>34</v>
@@ -47235,13 +47295,13 @@
         <v>3</v>
       </c>
       <c r="C417" s="30" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="D417" s="30" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="E417" s="37" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="F417" s="31" t="s">
         <v>30</v>
@@ -47318,13 +47378,13 @@
         <v>3</v>
       </c>
       <c r="C418" s="30" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="D418" s="30" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="E418" s="37" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="F418" s="31" t="s">
         <v>26</v>
@@ -47401,13 +47461,13 @@
         <v>3</v>
       </c>
       <c r="C419" s="30" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="D419" s="30" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="E419" s="37" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="F419" s="31" t="s">
         <v>22</v>
@@ -47484,13 +47544,13 @@
         <v>3</v>
       </c>
       <c r="C420" s="30" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="D420" s="30" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="E420" s="37" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="F420" s="31" t="s">
         <v>55</v>
@@ -47567,13 +47627,13 @@
         <v>3</v>
       </c>
       <c r="C421" s="30" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="D421" s="30" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="E421" s="37" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="F421" s="31" t="s">
         <v>59</v>
@@ -47650,16 +47710,16 @@
         <v>3</v>
       </c>
       <c r="C422" s="30" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="D422" s="30" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="E422" s="37" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="F422" s="31" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="G422" s="30">
         <v>48</v>
@@ -48224,7 +48284,7 @@
         <v>263</v>
       </c>
       <c r="E426" s="52" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="F426" s="30"/>
       <c r="G426" s="30">
@@ -48411,7 +48471,7 @@
         <v>264</v>
       </c>
       <c r="E427" s="52" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="F427" s="30"/>
       <c r="G427" s="30">

</xml_diff>